<commit_message>
Upgraded "2D Diagram for Ig Domains" to have one diagram for each Ig domain in a chain.
</commit_message>
<xml_diff>
--- a/template/igstrand_template_IgC1.xlsx
+++ b/template/igstrand_template_IgC1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nih-my.sharepoint.com/personal/khaniyau2_nih_gov/Documents/_Data/project_ig_survey/igstrand_tmalign/paper_2d_mapping/code/input/igstrand_template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangjiy\Documents\webgl\2D-template\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{411BA149-1EDC-C14E-801F-53D5C994A2CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1771EEC-EEEF-2C41-8544-3609A49780C6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79567100-5512-4379-B297-712460BDD1CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2600" yWindow="760" windowWidth="27640" windowHeight="16940" xr2:uid="{82E70425-45EB-014A-A1A7-8718A7FA18C9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{82E70425-45EB-014A-A1A7-8718A7FA18C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,12 +36,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="35">
   <si>
     <t>NUMBERING</t>
-  </si>
-  <si>
-    <t>C1 domain</t>
   </si>
   <si>
     <t>7-Strands</t>
@@ -125,9 +122,6 @@
     <t>*</t>
   </si>
   <si>
-    <t>CHECK</t>
-  </si>
-  <si>
     <t>HV4</t>
   </si>
   <si>
@@ -146,7 +140,7 @@
     <t>Nt</t>
   </si>
   <si>
-    <t>D strand 6555 65556?</t>
+    <t>IgC1</t>
   </si>
 </sst>
 </file>
@@ -240,7 +234,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -343,6 +337,12 @@
         <bgColor rgb="FFEFEFEF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="9">
     <border>
@@ -432,7 +432,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -616,6 +616,7 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -968,18 +969,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3908B27F-B803-2846-8197-EBED9FE0C8A9}">
-  <dimension ref="A1:Y329"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <dimension ref="A1:S329"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="3" width="4.33203125" customWidth="1"/>
-    <col min="4" max="6" width="6.1640625" customWidth="1"/>
-    <col min="7" max="11" width="6.33203125" customWidth="1"/>
-    <col min="12" max="14" width="7.1640625" customWidth="1"/>
-    <col min="15" max="19" width="4.33203125" customWidth="1"/>
-    <col min="21" max="21" width="12.1640625" customWidth="1"/>
+    <col min="1" max="3" width="4.375" customWidth="1"/>
+    <col min="4" max="6" width="6.125" customWidth="1"/>
+    <col min="7" max="11" width="6.375" customWidth="1"/>
+    <col min="12" max="14" width="7.125" customWidth="1"/>
+    <col min="15" max="19" width="4.375" customWidth="1"/>
+    <col min="21" max="21" width="12.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="20">
+    <row r="1" spans="1:19" ht="20.25">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -991,7 +992,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="2" t="s">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -999,7 +1000,7 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
       <c r="O1" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
@@ -1033,7 +1034,7 @@
       <c r="C3" s="4"/>
       <c r="D3" s="5"/>
       <c r="E3" s="6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="7"/>
@@ -1043,7 +1044,7 @@
       <c r="K3" s="4"/>
       <c r="L3" s="8"/>
       <c r="M3" s="9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N3" s="8"/>
       <c r="O3" s="4"/>
@@ -1057,29 +1058,29 @@
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
       <c r="D4" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="F4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="G4" s="11" t="s">
         <v>7</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>8</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="M4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="M4" s="11" t="s">
+      <c r="N4" s="10" t="s">
         <v>10</v>
-      </c>
-      <c r="N4" s="10" t="s">
-        <v>11</v>
       </c>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
@@ -1092,29 +1093,29 @@
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="12" t="s">
-        <v>13</v>
-      </c>
       <c r="F5" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="11" t="s">
         <v>12</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>13</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="M5" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="M5" s="13" t="s">
-        <v>13</v>
-      </c>
       <c r="N5" s="12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
@@ -1122,34 +1123,34 @@
       <c r="R5" s="4"/>
       <c r="S5" s="3"/>
     </row>
-    <row r="6" spans="1:19" ht="20">
+    <row r="6" spans="1:19" ht="20.25">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="F6" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="G6" s="17" t="s">
         <v>16</v>
-      </c>
-      <c r="G6" s="17" t="s">
-        <v>17</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="M6" s="19" t="s">
+      <c r="N6" s="20" t="s">
         <v>19</v>
-      </c>
-      <c r="N6" s="20" t="s">
-        <v>20</v>
       </c>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
@@ -1205,7 +1206,7 @@
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
       <c r="L8" s="28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
@@ -1215,24 +1216,24 @@
       <c r="R8" s="4"/>
       <c r="S8" s="3"/>
     </row>
-    <row r="9" spans="1:19" ht="17" thickBot="1">
+    <row r="9" spans="1:19" ht="16.5" thickBot="1">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
-      <c r="D9" s="81" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="78"/>
+      <c r="D9" s="82" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="79"/>
       <c r="F9" s="4"/>
       <c r="G9" s="29"/>
       <c r="H9" s="29"/>
-      <c r="I9" s="82" t="s">
-        <v>23</v>
-      </c>
-      <c r="J9" s="83"/>
+      <c r="I9" s="83" t="s">
+        <v>22</v>
+      </c>
+      <c r="J9" s="84"/>
       <c r="K9" s="30"/>
       <c r="L9" s="31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M9" s="29"/>
       <c r="N9" s="29"/>
@@ -1242,7 +1243,7 @@
       <c r="R9" s="4"/>
       <c r="S9" s="3"/>
     </row>
-    <row r="10" spans="1:19" ht="18" thickTop="1" thickBot="1">
+    <row r="10" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1260,7 +1261,7 @@
         <v>6544</v>
       </c>
       <c r="K10" s="33" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L10" s="33">
         <v>3559</v>
@@ -1275,7 +1276,7 @@
       <c r="R10" s="4"/>
       <c r="S10" s="3"/>
     </row>
-    <row r="11" spans="1:19" ht="18" thickTop="1" thickBot="1">
+    <row r="11" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1284,10 +1285,10 @@
       <c r="F11" s="30"/>
       <c r="G11" s="30"/>
       <c r="H11" s="29"/>
-      <c r="I11" s="82" t="s">
-        <v>25</v>
-      </c>
-      <c r="J11" s="83"/>
+      <c r="I11" s="83" t="s">
+        <v>24</v>
+      </c>
+      <c r="J11" s="84"/>
       <c r="K11" s="30"/>
       <c r="L11" s="34"/>
       <c r="M11" s="30"/>
@@ -1298,15 +1299,15 @@
       <c r="R11" s="4"/>
       <c r="S11" s="3"/>
     </row>
-    <row r="12" spans="1:19" ht="18" thickTop="1" thickBot="1">
+    <row r="12" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="32"/>
       <c r="D12" s="35" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="33">
@@ -1316,7 +1317,7 @@
         <v>7556</v>
       </c>
       <c r="I12" s="33" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J12" s="33">
         <v>8542</v>
@@ -1325,7 +1326,7 @@
         <v>8543</v>
       </c>
       <c r="L12" s="33" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M12" s="32"/>
       <c r="N12" s="32"/>
@@ -1335,7 +1336,7 @@
       <c r="R12" s="4"/>
       <c r="S12" s="3"/>
     </row>
-    <row r="13" spans="1:19" ht="17" thickTop="1">
+    <row r="13" spans="1:19" ht="16.5" thickTop="1">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="32"/>
@@ -1459,7 +1460,7 @@
       <c r="R16" s="4"/>
       <c r="S16" s="3"/>
     </row>
-    <row r="17" spans="1:25">
+    <row r="17" spans="1:19">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="32"/>
@@ -1494,7 +1495,7 @@
       <c r="R17" s="4"/>
       <c r="S17" s="3"/>
     </row>
-    <row r="18" spans="1:25">
+    <row r="18" spans="1:19">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
       <c r="C18" s="32"/>
@@ -1529,7 +1530,7 @@
       <c r="R18" s="4"/>
       <c r="S18" s="3"/>
     </row>
-    <row r="19" spans="1:25">
+    <row r="19" spans="1:19">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="32"/>
@@ -1556,7 +1557,7 @@
       <c r="R19" s="4"/>
       <c r="S19" s="3"/>
     </row>
-    <row r="20" spans="1:25">
+    <row r="20" spans="1:19">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="32"/>
@@ -1590,11 +1591,8 @@
       <c r="Q20" s="4"/>
       <c r="R20" s="4"/>
       <c r="S20" s="3"/>
-      <c r="Y20" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="21" spans="1:25">
+    </row>
+    <row r="21" spans="1:19">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="32"/>
@@ -1625,7 +1623,7 @@
       <c r="R21" s="4"/>
       <c r="S21" s="3"/>
     </row>
-    <row r="22" spans="1:25">
+    <row r="22" spans="1:19">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="C22" s="32"/>
@@ -1642,12 +1640,12 @@
         <v>6552</v>
       </c>
       <c r="H22" s="61" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I22" s="62"/>
       <c r="J22" s="62"/>
       <c r="K22" s="63" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L22" s="41">
         <v>9550</v>
@@ -1664,7 +1662,7 @@
       <c r="R22" s="4"/>
       <c r="S22" s="3"/>
     </row>
-    <row r="23" spans="1:25">
+    <row r="23" spans="1:19">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="C23" s="32"/>
@@ -1685,13 +1683,13 @@
       <c r="L23" s="64"/>
       <c r="M23" s="59"/>
       <c r="N23" s="60"/>
-      <c r="O23" s="62"/>
-      <c r="P23" s="62"/>
-      <c r="Q23" s="62"/>
+      <c r="O23" s="77"/>
+      <c r="P23" s="77"/>
+      <c r="Q23" s="77"/>
       <c r="R23" s="4"/>
       <c r="S23" s="3"/>
     </row>
-    <row r="24" spans="1:25">
+    <row r="24" spans="1:19">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="C24" s="32"/>
@@ -1720,15 +1718,13 @@
       <c r="N24" s="53">
         <v>3549</v>
       </c>
-      <c r="O24" s="62"/>
-      <c r="P24" s="62" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q24" s="62"/>
+      <c r="O24" s="77"/>
+      <c r="P24" s="77"/>
+      <c r="Q24" s="77"/>
       <c r="R24" s="4"/>
       <c r="S24" s="3"/>
     </row>
-    <row r="25" spans="1:25">
+    <row r="25" spans="1:19">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="C25" s="32"/>
@@ -1757,13 +1753,13 @@
       <c r="N25" s="53">
         <v>3548</v>
       </c>
-      <c r="O25" s="62"/>
-      <c r="P25" s="62"/>
-      <c r="Q25" s="62"/>
+      <c r="O25" s="77"/>
+      <c r="P25" s="77"/>
+      <c r="Q25" s="77"/>
       <c r="R25" s="4"/>
       <c r="S25" s="3"/>
     </row>
-    <row r="26" spans="1:25" ht="17" thickBot="1">
+    <row r="26" spans="1:19" ht="16.5" thickBot="1">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="C26" s="32"/>
@@ -1772,10 +1768,10 @@
       </c>
       <c r="E26" s="55"/>
       <c r="F26" s="67" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G26" s="68" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
@@ -1790,13 +1786,13 @@
       <c r="N26" s="53">
         <v>3547</v>
       </c>
-      <c r="O26" s="62"/>
-      <c r="P26" s="62"/>
-      <c r="Q26" s="62"/>
+      <c r="O26" s="77"/>
+      <c r="P26" s="77"/>
+      <c r="Q26" s="77"/>
       <c r="R26" s="4"/>
       <c r="S26" s="3"/>
     </row>
-    <row r="27" spans="1:25" ht="17" thickTop="1">
+    <row r="27" spans="1:19" ht="16.5" thickTop="1">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
       <c r="C27" s="32"/>
@@ -1806,10 +1802,10 @@
       <c r="E27" s="66">
         <v>2554</v>
       </c>
-      <c r="F27" s="77" t="s">
-        <v>24</v>
-      </c>
-      <c r="G27" s="78"/>
+      <c r="F27" s="78" t="s">
+        <v>23</v>
+      </c>
+      <c r="G27" s="79"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
@@ -1829,7 +1825,7 @@
       <c r="R27" s="4"/>
       <c r="S27" s="3"/>
     </row>
-    <row r="28" spans="1:25" ht="17" thickBot="1">
+    <row r="28" spans="1:19" ht="16.5" thickBot="1">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
       <c r="C28" s="32"/>
@@ -1839,19 +1835,19 @@
       <c r="E28" s="66">
         <v>2555</v>
       </c>
-      <c r="F28" s="84" t="s">
-        <v>30</v>
-      </c>
-      <c r="G28" s="78"/>
+      <c r="F28" s="85" t="s">
+        <v>28</v>
+      </c>
+      <c r="G28" s="79"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
       <c r="K28" s="32"/>
       <c r="L28" s="71" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="M28" s="72" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="N28" s="66">
         <v>3545</v>
@@ -1862,7 +1858,7 @@
       <c r="R28" s="4"/>
       <c r="S28" s="3"/>
     </row>
-    <row r="29" spans="1:25" ht="18" thickTop="1" thickBot="1">
+    <row r="29" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
       <c r="C29" s="32"/>
@@ -1883,14 +1879,14 @@
       <c r="R29" s="4"/>
       <c r="S29" s="3"/>
     </row>
-    <row r="30" spans="1:25" ht="18" thickTop="1" thickBot="1">
+    <row r="30" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
       <c r="C30" s="32"/>
       <c r="D30" s="73"/>
       <c r="E30" s="74"/>
       <c r="F30" s="67" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G30" s="67">
         <v>2556</v>
@@ -1911,7 +1907,7 @@
         <v>3544</v>
       </c>
       <c r="M30" s="67" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N30" s="34"/>
       <c r="O30" s="4"/>
@@ -1920,26 +1916,26 @@
       <c r="R30" s="4"/>
       <c r="S30" s="3"/>
     </row>
-    <row r="31" spans="1:25" ht="17" thickTop="1">
+    <row r="31" spans="1:19" ht="16.5" thickTop="1">
       <c r="A31" s="3"/>
       <c r="B31" s="4"/>
       <c r="C31" s="32"/>
       <c r="D31" s="73"/>
       <c r="E31" s="4"/>
-      <c r="F31" s="77" t="s">
-        <v>24</v>
-      </c>
-      <c r="G31" s="78"/>
+      <c r="F31" s="78" t="s">
+        <v>23</v>
+      </c>
+      <c r="G31" s="79"/>
       <c r="H31" s="4"/>
-      <c r="I31" s="79" t="s">
-        <v>32</v>
-      </c>
-      <c r="J31" s="78"/>
+      <c r="I31" s="80" t="s">
+        <v>30</v>
+      </c>
+      <c r="J31" s="79"/>
       <c r="K31" s="4"/>
-      <c r="L31" s="77" t="s">
-        <v>24</v>
-      </c>
-      <c r="M31" s="78"/>
+      <c r="L31" s="78" t="s">
+        <v>23</v>
+      </c>
+      <c r="M31" s="79"/>
       <c r="N31" s="4"/>
       <c r="O31" s="4"/>
       <c r="P31" s="4"/>
@@ -1947,24 +1943,24 @@
       <c r="R31" s="4"/>
       <c r="S31" s="3"/>
     </row>
-    <row r="32" spans="1:25">
+    <row r="32" spans="1:19">
       <c r="A32" s="3"/>
       <c r="B32" s="4"/>
       <c r="C32" s="32"/>
       <c r="D32" s="73"/>
       <c r="E32" s="4"/>
-      <c r="F32" s="79" t="s">
-        <v>33</v>
-      </c>
-      <c r="G32" s="78"/>
+      <c r="F32" s="80" t="s">
+        <v>31</v>
+      </c>
+      <c r="G32" s="79"/>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
-      <c r="L32" s="79" t="s">
-        <v>34</v>
-      </c>
-      <c r="M32" s="78"/>
+      <c r="L32" s="80" t="s">
+        <v>32</v>
+      </c>
+      <c r="M32" s="79"/>
       <c r="N32" s="4"/>
       <c r="O32" s="4"/>
       <c r="P32" s="4"/>
@@ -1998,13 +1994,13 @@
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
-      <c r="H34" s="80"/>
-      <c r="I34" s="78"/>
+      <c r="H34" s="81"/>
+      <c r="I34" s="79"/>
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
@@ -2021,7 +2017,7 @@
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="28" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
@@ -2228,7 +2224,7 @@
       <c r="R44" s="4"/>
       <c r="S44" s="3"/>
     </row>
-    <row r="45" spans="1:19" ht="17" thickBot="1">
+    <row r="45" spans="1:19" ht="16.5" thickBot="1">
       <c r="A45" s="75"/>
       <c r="B45" s="75"/>
       <c r="C45" s="75"/>

</xml_diff>

<commit_message>
Updated "2D Diagram for Nucleotides" so that users can click on 2D Diagram to show selection on 3D view.
</commit_message>
<xml_diff>
--- a/template/igstrand_template_IgC1.xlsx
+++ b/template/igstrand_template_IgC1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangjiy\Documents\webgl\2D-template\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79567100-5512-4379-B297-712460BDD1CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715BF52C-AF78-49FA-BAF1-25D03AE88484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{82E70425-45EB-014A-A1A7-8718A7FA18C9}"/>
   </bookViews>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="35">
-  <si>
-    <t>NUMBERING</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="36">
   <si>
     <t>7-Strands</t>
   </si>
@@ -101,9 +98,6 @@
     <t>Ct</t>
   </si>
   <si>
-    <t>A-B</t>
-  </si>
-  <si>
     <t>C"-D</t>
   </si>
   <si>
@@ -141,6 +135,15 @@
   </si>
   <si>
     <t>IgC1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       A-B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       ←</t>
+  </si>
+  <si>
+    <t>NUMBERING</t>
   </si>
 </sst>
 </file>
@@ -620,21 +623,21 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -969,21 +972,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3908B27F-B803-2846-8197-EBED9FE0C8A9}">
-  <dimension ref="A1:S329"/>
+  <dimension ref="A1:Q324"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="3" width="4.375" customWidth="1"/>
-    <col min="4" max="6" width="6.125" customWidth="1"/>
-    <col min="7" max="11" width="6.375" customWidth="1"/>
-    <col min="12" max="14" width="7.125" customWidth="1"/>
-    <col min="15" max="19" width="4.375" customWidth="1"/>
-    <col min="21" max="21" width="12.125" customWidth="1"/>
+    <col min="4" max="4" width="7.375" customWidth="1"/>
+    <col min="5" max="5" width="7.5" customWidth="1"/>
+    <col min="6" max="6" width="7" customWidth="1"/>
+    <col min="7" max="7" width="7.375" customWidth="1"/>
+    <col min="8" max="11" width="6.375" customWidth="1"/>
+    <col min="12" max="12" width="7.125" customWidth="1"/>
+    <col min="13" max="13" width="7.5" customWidth="1"/>
+    <col min="14" max="14" width="7.875" customWidth="1"/>
+    <col min="15" max="17" width="4.375" customWidth="1"/>
+    <col min="19" max="19" width="12.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="20.25">
+    <row r="1" spans="1:17" ht="20.25">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -992,7 +1000,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -1000,14 +1008,12 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
       <c r="O1" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-    </row>
-    <row r="2" spans="1:19">
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" s="3"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -1024,17 +1030,15 @@
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="3"/>
-    </row>
-    <row r="3" spans="1:19">
+      <c r="Q2" s="3"/>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="5"/>
       <c r="E3" s="6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="7"/>
@@ -1044,121 +1048,113 @@
       <c r="K3" s="4"/>
       <c r="L3" s="8"/>
       <c r="M3" s="9" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N3" s="8"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="3"/>
-    </row>
-    <row r="4" spans="1:19">
+      <c r="Q3" s="3"/>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
       <c r="D4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="F4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="G4" s="11" t="s">
         <v>6</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>7</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="M4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="M4" s="11" t="s">
+      <c r="N4" s="10" t="s">
         <v>9</v>
-      </c>
-      <c r="N4" s="10" t="s">
-        <v>10</v>
       </c>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="3"/>
-    </row>
-    <row r="5" spans="1:19">
+      <c r="Q4" s="3"/>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="12" t="s">
-        <v>12</v>
-      </c>
       <c r="F5" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="11" t="s">
         <v>11</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>12</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="M5" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="M5" s="13" t="s">
-        <v>12</v>
-      </c>
       <c r="N5" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="3"/>
-    </row>
-    <row r="6" spans="1:19" ht="20.25">
+      <c r="Q5" s="3"/>
+    </row>
+    <row r="6" spans="1:17" ht="20.25">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="F6" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="G6" s="17" t="s">
         <v>15</v>
-      </c>
-      <c r="G6" s="17" t="s">
-        <v>16</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="M6" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="M6" s="19" t="s">
+      <c r="N6" s="20" t="s">
         <v>18</v>
-      </c>
-      <c r="N6" s="20" t="s">
-        <v>19</v>
       </c>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
-      <c r="Q6" s="4"/>
-      <c r="R6" s="4"/>
-      <c r="S6" s="3"/>
-    </row>
-    <row r="7" spans="1:19">
+      <c r="Q6" s="3"/>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1189,11 +1185,9 @@
       </c>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
-      <c r="Q7" s="4"/>
-      <c r="R7" s="4"/>
-      <c r="S7" s="3"/>
-    </row>
-    <row r="8" spans="1:19">
+      <c r="Q7" s="3"/>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1206,44 +1200,39 @@
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
       <c r="L8" s="28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
-      <c r="Q8" s="4"/>
-      <c r="R8" s="4"/>
-      <c r="S8" s="3"/>
-    </row>
-    <row r="9" spans="1:19" ht="16.5" thickBot="1">
+      <c r="Q8" s="3"/>
+    </row>
+    <row r="9" spans="1:17" ht="16.5" thickBot="1">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
-      <c r="D9" s="82" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="79"/>
+      <c r="D9" s="80" t="s">
+        <v>33</v>
+      </c>
       <c r="F9" s="4"/>
       <c r="G9" s="29"/>
       <c r="H9" s="29"/>
-      <c r="I9" s="83" t="s">
-        <v>22</v>
-      </c>
-      <c r="J9" s="84"/>
+      <c r="I9" s="81" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9" s="83"/>
       <c r="K9" s="30"/>
       <c r="L9" s="31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M9" s="29"/>
       <c r="N9" s="29"/>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
-      <c r="Q9" s="4"/>
-      <c r="R9" s="4"/>
-      <c r="S9" s="3"/>
-    </row>
-    <row r="10" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
+      <c r="Q9" s="3"/>
+    </row>
+    <row r="10" spans="1:17" ht="17.25" thickTop="1" thickBot="1">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1261,7 +1250,7 @@
         <v>6544</v>
       </c>
       <c r="K10" s="33" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L10" s="33">
         <v>3559</v>
@@ -1272,11 +1261,9 @@
       <c r="N10" s="32"/>
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
-      <c r="Q10" s="4"/>
-      <c r="R10" s="4"/>
-      <c r="S10" s="3"/>
-    </row>
-    <row r="11" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
+      <c r="Q10" s="3"/>
+    </row>
+    <row r="11" spans="1:17" ht="17.25" thickTop="1" thickBot="1">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1285,29 +1272,27 @@
       <c r="F11" s="30"/>
       <c r="G11" s="30"/>
       <c r="H11" s="29"/>
-      <c r="I11" s="83" t="s">
-        <v>24</v>
-      </c>
-      <c r="J11" s="84"/>
+      <c r="I11" s="81" t="s">
+        <v>22</v>
+      </c>
+      <c r="J11" s="83"/>
       <c r="K11" s="30"/>
       <c r="L11" s="34"/>
       <c r="M11" s="30"/>
       <c r="N11" s="32"/>
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
-      <c r="Q11" s="4"/>
-      <c r="R11" s="4"/>
-      <c r="S11" s="3"/>
-    </row>
-    <row r="12" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
+      <c r="Q11" s="3"/>
+    </row>
+    <row r="12" spans="1:17" ht="17.25" thickTop="1" thickBot="1">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="32"/>
       <c r="D12" s="35" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="33">
@@ -1317,7 +1302,7 @@
         <v>7556</v>
       </c>
       <c r="I12" s="33" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J12" s="33">
         <v>8542</v>
@@ -1326,17 +1311,15 @@
         <v>8543</v>
       </c>
       <c r="L12" s="33" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M12" s="32"/>
       <c r="N12" s="32"/>
       <c r="O12" s="4"/>
       <c r="P12" s="4"/>
-      <c r="Q12" s="4"/>
-      <c r="R12" s="4"/>
-      <c r="S12" s="3"/>
-    </row>
-    <row r="13" spans="1:19" ht="16.5" thickTop="1">
+      <c r="Q12" s="3"/>
+    </row>
+    <row r="13" spans="1:17" ht="16.5" thickTop="1">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="32"/>
@@ -1361,11 +1344,9 @@
       <c r="N13" s="32"/>
       <c r="O13" s="4"/>
       <c r="P13" s="4"/>
-      <c r="Q13" s="4"/>
-      <c r="R13" s="4"/>
-      <c r="S13" s="3"/>
-    </row>
-    <row r="14" spans="1:19">
+      <c r="Q13" s="3"/>
+    </row>
+    <row r="14" spans="1:17">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="32"/>
@@ -1390,11 +1371,9 @@
       </c>
       <c r="O14" s="4"/>
       <c r="P14" s="4"/>
-      <c r="Q14" s="4"/>
-      <c r="R14" s="4"/>
-      <c r="S14" s="3"/>
-    </row>
-    <row r="15" spans="1:19">
+      <c r="Q14" s="3"/>
+    </row>
+    <row r="15" spans="1:17">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="32"/>
@@ -1421,11 +1400,9 @@
       </c>
       <c r="O15" s="4"/>
       <c r="P15" s="4"/>
-      <c r="Q15" s="4"/>
-      <c r="R15" s="4"/>
-      <c r="S15" s="3"/>
-    </row>
-    <row r="16" spans="1:19">
+      <c r="Q15" s="3"/>
+    </row>
+    <row r="16" spans="1:17">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="32"/>
@@ -1456,11 +1433,9 @@
       </c>
       <c r="O16" s="4"/>
       <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
-      <c r="R16" s="4"/>
-      <c r="S16" s="3"/>
-    </row>
-    <row r="17" spans="1:19">
+      <c r="Q16" s="3"/>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="32"/>
@@ -1491,11 +1466,9 @@
       </c>
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
-      <c r="Q17" s="4"/>
-      <c r="R17" s="4"/>
-      <c r="S17" s="3"/>
-    </row>
-    <row r="18" spans="1:19">
+      <c r="Q17" s="3"/>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
       <c r="C18" s="32"/>
@@ -1526,11 +1499,9 @@
       </c>
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
-      <c r="Q18" s="4"/>
-      <c r="R18" s="4"/>
-      <c r="S18" s="3"/>
-    </row>
-    <row r="19" spans="1:19">
+      <c r="Q18" s="3"/>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="32"/>
@@ -1553,11 +1524,9 @@
       </c>
       <c r="O19" s="4"/>
       <c r="P19" s="4"/>
-      <c r="Q19" s="4"/>
-      <c r="R19" s="4"/>
-      <c r="S19" s="3"/>
-    </row>
-    <row r="20" spans="1:19">
+      <c r="Q19" s="3"/>
+    </row>
+    <row r="20" spans="1:17">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="32"/>
@@ -1588,11 +1557,9 @@
       </c>
       <c r="O20" s="4"/>
       <c r="P20" s="4"/>
-      <c r="Q20" s="4"/>
-      <c r="R20" s="4"/>
-      <c r="S20" s="3"/>
-    </row>
-    <row r="21" spans="1:19">
+      <c r="Q20" s="3"/>
+    </row>
+    <row r="21" spans="1:17">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="32"/>
@@ -1619,11 +1586,9 @@
       <c r="N21" s="60"/>
       <c r="O21" s="4"/>
       <c r="P21" s="4"/>
-      <c r="Q21" s="4"/>
-      <c r="R21" s="4"/>
-      <c r="S21" s="3"/>
-    </row>
-    <row r="22" spans="1:19">
+      <c r="Q21" s="3"/>
+    </row>
+    <row r="22" spans="1:17">
       <c r="A22" s="3"/>
       <c r="B22" s="4"/>
       <c r="C22" s="32"/>
@@ -1640,12 +1605,12 @@
         <v>6552</v>
       </c>
       <c r="H22" s="61" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I22" s="62"/>
       <c r="J22" s="62"/>
       <c r="K22" s="63" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="L22" s="41">
         <v>9550</v>
@@ -1658,11 +1623,9 @@
       </c>
       <c r="O22" s="4"/>
       <c r="P22" s="4"/>
-      <c r="Q22" s="4"/>
-      <c r="R22" s="4"/>
-      <c r="S22" s="3"/>
-    </row>
-    <row r="23" spans="1:19">
+      <c r="Q22" s="3"/>
+    </row>
+    <row r="23" spans="1:17">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="C23" s="32"/>
@@ -1684,12 +1647,10 @@
       <c r="M23" s="59"/>
       <c r="N23" s="60"/>
       <c r="O23" s="77"/>
-      <c r="P23" s="77"/>
-      <c r="Q23" s="77"/>
-      <c r="R23" s="4"/>
-      <c r="S23" s="3"/>
-    </row>
-    <row r="24" spans="1:19">
+      <c r="P23" s="4"/>
+      <c r="Q23" s="3"/>
+    </row>
+    <row r="24" spans="1:17">
       <c r="A24" s="3"/>
       <c r="B24" s="4"/>
       <c r="C24" s="32"/>
@@ -1719,12 +1680,10 @@
         <v>3549</v>
       </c>
       <c r="O24" s="77"/>
-      <c r="P24" s="77"/>
-      <c r="Q24" s="77"/>
-      <c r="R24" s="4"/>
-      <c r="S24" s="3"/>
-    </row>
-    <row r="25" spans="1:19">
+      <c r="P24" s="4"/>
+      <c r="Q24" s="3"/>
+    </row>
+    <row r="25" spans="1:17">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
       <c r="C25" s="32"/>
@@ -1754,12 +1713,10 @@
         <v>3548</v>
       </c>
       <c r="O25" s="77"/>
-      <c r="P25" s="77"/>
-      <c r="Q25" s="77"/>
-      <c r="R25" s="4"/>
-      <c r="S25" s="3"/>
-    </row>
-    <row r="26" spans="1:19" ht="16.5" thickBot="1">
+      <c r="P25" s="4"/>
+      <c r="Q25" s="3"/>
+    </row>
+    <row r="26" spans="1:17" ht="16.5" thickBot="1">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
       <c r="C26" s="32"/>
@@ -1768,10 +1725,10 @@
       </c>
       <c r="E26" s="55"/>
       <c r="F26" s="67" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G26" s="68" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
@@ -1787,12 +1744,10 @@
         <v>3547</v>
       </c>
       <c r="O26" s="77"/>
-      <c r="P26" s="77"/>
-      <c r="Q26" s="77"/>
-      <c r="R26" s="4"/>
-      <c r="S26" s="3"/>
-    </row>
-    <row r="27" spans="1:19" ht="16.5" thickTop="1">
+      <c r="P26" s="4"/>
+      <c r="Q26" s="3"/>
+    </row>
+    <row r="27" spans="1:17" ht="16.5" thickTop="1">
       <c r="A27" s="3"/>
       <c r="B27" s="4"/>
       <c r="C27" s="32"/>
@@ -1803,9 +1758,9 @@
         <v>2554</v>
       </c>
       <c r="F27" s="78" t="s">
-        <v>23</v>
-      </c>
-      <c r="G27" s="79"/>
+        <v>34</v>
+      </c>
+      <c r="G27" s="4"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
@@ -1821,11 +1776,9 @@
       </c>
       <c r="O27" s="4"/>
       <c r="P27" s="4"/>
-      <c r="Q27" s="4"/>
-      <c r="R27" s="4"/>
-      <c r="S27" s="3"/>
-    </row>
-    <row r="28" spans="1:19" ht="16.5" thickBot="1">
+      <c r="Q27" s="3"/>
+    </row>
+    <row r="28" spans="1:17" ht="16.5" thickBot="1">
       <c r="A28" s="3"/>
       <c r="B28" s="4"/>
       <c r="C28" s="32"/>
@@ -1835,30 +1788,27 @@
       <c r="E28" s="66">
         <v>2555</v>
       </c>
-      <c r="F28" s="85" t="s">
-        <v>28</v>
-      </c>
-      <c r="G28" s="79"/>
+      <c r="F28" s="82" t="s">
+        <v>26</v>
+      </c>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
       <c r="K28" s="32"/>
       <c r="L28" s="71" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="M28" s="72" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="N28" s="66">
         <v>3545</v>
       </c>
       <c r="O28" s="4"/>
       <c r="P28" s="4"/>
-      <c r="Q28" s="4"/>
-      <c r="R28" s="4"/>
-      <c r="S28" s="3"/>
-    </row>
-    <row r="29" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
+      <c r="Q28" s="3"/>
+    </row>
+    <row r="29" spans="1:17" ht="17.25" thickTop="1" thickBot="1">
       <c r="A29" s="3"/>
       <c r="B29" s="4"/>
       <c r="C29" s="32"/>
@@ -1875,18 +1825,16 @@
       <c r="N29" s="73"/>
       <c r="O29" s="4"/>
       <c r="P29" s="4"/>
-      <c r="Q29" s="4"/>
-      <c r="R29" s="4"/>
-      <c r="S29" s="3"/>
-    </row>
-    <row r="30" spans="1:19" ht="17.25" thickTop="1" thickBot="1">
+      <c r="Q29" s="3"/>
+    </row>
+    <row r="30" spans="1:17" ht="17.25" thickTop="1" thickBot="1">
       <c r="A30" s="3"/>
       <c r="B30" s="4"/>
       <c r="C30" s="32"/>
       <c r="D30" s="73"/>
       <c r="E30" s="74"/>
       <c r="F30" s="67" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G30" s="67">
         <v>2556</v>
@@ -1907,68 +1855,59 @@
         <v>3544</v>
       </c>
       <c r="M30" s="67" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="N30" s="34"/>
       <c r="O30" s="4"/>
       <c r="P30" s="4"/>
-      <c r="Q30" s="4"/>
-      <c r="R30" s="4"/>
-      <c r="S30" s="3"/>
-    </row>
-    <row r="31" spans="1:19" ht="16.5" thickTop="1">
+      <c r="Q30" s="3"/>
+    </row>
+    <row r="31" spans="1:17" ht="16.5" thickTop="1">
       <c r="A31" s="3"/>
       <c r="B31" s="4"/>
       <c r="C31" s="32"/>
       <c r="D31" s="73"/>
       <c r="E31" s="4"/>
       <c r="F31" s="78" t="s">
-        <v>23</v>
-      </c>
-      <c r="G31" s="79"/>
+        <v>34</v>
+      </c>
+      <c r="G31" s="4"/>
       <c r="H31" s="4"/>
-      <c r="I31" s="80" t="s">
-        <v>30</v>
-      </c>
-      <c r="J31" s="79"/>
+      <c r="I31" s="79" t="s">
+        <v>28</v>
+      </c>
       <c r="K31" s="4"/>
       <c r="L31" s="78" t="s">
-        <v>23</v>
-      </c>
-      <c r="M31" s="79"/>
+        <v>34</v>
+      </c>
+      <c r="M31" s="4"/>
       <c r="N31" s="4"/>
       <c r="O31" s="4"/>
       <c r="P31" s="4"/>
-      <c r="Q31" s="4"/>
-      <c r="R31" s="4"/>
-      <c r="S31" s="3"/>
-    </row>
-    <row r="32" spans="1:19">
+      <c r="Q31" s="3"/>
+    </row>
+    <row r="32" spans="1:17">
       <c r="A32" s="3"/>
       <c r="B32" s="4"/>
       <c r="C32" s="32"/>
       <c r="D32" s="73"/>
       <c r="E32" s="4"/>
-      <c r="F32" s="80" t="s">
-        <v>31</v>
-      </c>
-      <c r="G32" s="79"/>
+      <c r="F32" s="79" t="s">
+        <v>29</v>
+      </c>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
-      <c r="L32" s="80" t="s">
-        <v>32</v>
-      </c>
-      <c r="M32" s="79"/>
+      <c r="L32" s="79" t="s">
+        <v>30</v>
+      </c>
       <c r="N32" s="4"/>
       <c r="O32" s="4"/>
       <c r="P32" s="4"/>
-      <c r="Q32" s="4"/>
-      <c r="R32" s="4"/>
-      <c r="S32" s="3"/>
-    </row>
-    <row r="33" spans="1:19">
+      <c r="Q32" s="3"/>
+    </row>
+    <row r="33" spans="1:17">
       <c r="A33" s="3"/>
       <c r="B33" s="4"/>
       <c r="C33" s="32"/>
@@ -1985,22 +1924,20 @@
       <c r="N33" s="4"/>
       <c r="O33" s="4"/>
       <c r="P33" s="4"/>
-      <c r="Q33" s="4"/>
-      <c r="R33" s="4"/>
-      <c r="S33" s="3"/>
-    </row>
-    <row r="34" spans="1:19">
+      <c r="Q33" s="3"/>
+    </row>
+    <row r="34" spans="1:17">
       <c r="A34" s="3"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
-      <c r="H34" s="81"/>
-      <c r="I34" s="79"/>
+      <c r="H34" s="84"/>
+      <c r="I34" s="85"/>
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
@@ -2008,20 +1945,17 @@
       <c r="N34" s="4"/>
       <c r="O34" s="4"/>
       <c r="P34" s="4"/>
-      <c r="Q34" s="4"/>
-      <c r="R34" s="4"/>
-      <c r="S34" s="3"/>
-    </row>
-    <row r="35" spans="1:19">
+      <c r="Q34" s="3"/>
+    </row>
+    <row r="35" spans="1:17">
       <c r="A35" s="3"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="28" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
@@ -2031,11 +1965,9 @@
       <c r="N35" s="4"/>
       <c r="O35" s="4"/>
       <c r="P35" s="4"/>
-      <c r="Q35" s="4"/>
-      <c r="R35" s="4"/>
-      <c r="S35" s="3"/>
-    </row>
-    <row r="36" spans="1:19">
+      <c r="Q35" s="3"/>
+    </row>
+    <row r="36" spans="1:17">
       <c r="A36" s="3"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -2052,11 +1984,9 @@
       <c r="N36" s="4"/>
       <c r="O36" s="4"/>
       <c r="P36" s="4"/>
-      <c r="Q36" s="4"/>
-      <c r="R36" s="4"/>
-      <c r="S36" s="3"/>
-    </row>
-    <row r="37" spans="1:19">
+      <c r="Q36" s="3"/>
+    </row>
+    <row r="37" spans="1:17">
       <c r="A37" s="3"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -2073,11 +2003,9 @@
       <c r="N37" s="4"/>
       <c r="O37" s="4"/>
       <c r="P37" s="4"/>
-      <c r="Q37" s="4"/>
-      <c r="R37" s="4"/>
-      <c r="S37" s="3"/>
-    </row>
-    <row r="38" spans="1:19">
+      <c r="Q37" s="3"/>
+    </row>
+    <row r="38" spans="1:17">
       <c r="A38" s="3"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -2094,11 +2022,9 @@
       <c r="N38" s="4"/>
       <c r="O38" s="4"/>
       <c r="P38" s="4"/>
-      <c r="Q38" s="4"/>
-      <c r="R38" s="4"/>
-      <c r="S38" s="3"/>
-    </row>
-    <row r="39" spans="1:19">
+      <c r="Q38" s="3"/>
+    </row>
+    <row r="39" spans="1:17">
       <c r="A39" s="3"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -2115,33 +2041,29 @@
       <c r="N39" s="4"/>
       <c r="O39" s="4"/>
       <c r="P39" s="4"/>
-      <c r="Q39" s="4"/>
-      <c r="R39" s="4"/>
-      <c r="S39" s="3"/>
-    </row>
-    <row r="40" spans="1:19">
-      <c r="A40" s="3"/>
-      <c r="B40" s="4"/>
-      <c r="C40" s="4"/>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
-      <c r="I40" s="4"/>
-      <c r="J40" s="4"/>
-      <c r="K40" s="4"/>
-      <c r="L40" s="4"/>
-      <c r="M40" s="4"/>
-      <c r="N40" s="4"/>
-      <c r="O40" s="4"/>
-      <c r="P40" s="4"/>
-      <c r="Q40" s="4"/>
-      <c r="R40" s="4"/>
-      <c r="S40" s="3"/>
-    </row>
-    <row r="41" spans="1:19">
-      <c r="A41" s="3"/>
+      <c r="Q39" s="3"/>
+    </row>
+    <row r="40" spans="1:17" ht="16.5" thickBot="1">
+      <c r="A40" s="75"/>
+      <c r="B40" s="75"/>
+      <c r="C40" s="75"/>
+      <c r="D40" s="75"/>
+      <c r="E40" s="75"/>
+      <c r="F40" s="75"/>
+      <c r="G40" s="75"/>
+      <c r="H40" s="75"/>
+      <c r="I40" s="75"/>
+      <c r="J40" s="75"/>
+      <c r="K40" s="75"/>
+      <c r="L40" s="75"/>
+      <c r="M40" s="75"/>
+      <c r="N40" s="75"/>
+      <c r="O40" s="75"/>
+      <c r="P40" s="75"/>
+      <c r="Q40" s="75"/>
+    </row>
+    <row r="41" spans="1:17">
+      <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
@@ -2158,11 +2080,9 @@
       <c r="O41" s="4"/>
       <c r="P41" s="4"/>
       <c r="Q41" s="4"/>
-      <c r="R41" s="4"/>
-      <c r="S41" s="3"/>
-    </row>
-    <row r="42" spans="1:19">
-      <c r="A42" s="3"/>
+    </row>
+    <row r="42" spans="1:17">
+      <c r="A42" s="4"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
@@ -2179,11 +2099,9 @@
       <c r="O42" s="4"/>
       <c r="P42" s="4"/>
       <c r="Q42" s="4"/>
-      <c r="R42" s="4"/>
-      <c r="S42" s="3"/>
-    </row>
-    <row r="43" spans="1:19">
-      <c r="A43" s="3"/>
+    </row>
+    <row r="43" spans="1:17">
+      <c r="A43" s="4"/>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
@@ -2200,11 +2118,9 @@
       <c r="O43" s="4"/>
       <c r="P43" s="4"/>
       <c r="Q43" s="4"/>
-      <c r="R43" s="4"/>
-      <c r="S43" s="3"/>
-    </row>
-    <row r="44" spans="1:19">
-      <c r="A44" s="3"/>
+    </row>
+    <row r="44" spans="1:17">
+      <c r="A44" s="4"/>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
@@ -2221,31 +2137,27 @@
       <c r="O44" s="4"/>
       <c r="P44" s="4"/>
       <c r="Q44" s="4"/>
-      <c r="R44" s="4"/>
-      <c r="S44" s="3"/>
-    </row>
-    <row r="45" spans="1:19" ht="16.5" thickBot="1">
-      <c r="A45" s="75"/>
-      <c r="B45" s="75"/>
-      <c r="C45" s="75"/>
-      <c r="D45" s="75"/>
-      <c r="E45" s="75"/>
-      <c r="F45" s="75"/>
-      <c r="G45" s="75"/>
-      <c r="H45" s="75"/>
-      <c r="I45" s="75"/>
-      <c r="J45" s="75"/>
-      <c r="K45" s="75"/>
-      <c r="L45" s="75"/>
-      <c r="M45" s="75"/>
-      <c r="N45" s="75"/>
-      <c r="O45" s="75"/>
-      <c r="P45" s="75"/>
-      <c r="Q45" s="75"/>
-      <c r="R45" s="75"/>
-      <c r="S45" s="75"/>
-    </row>
-    <row r="46" spans="1:19">
+    </row>
+    <row r="45" spans="1:17">
+      <c r="A45" s="4"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
+      <c r="I45" s="4"/>
+      <c r="J45" s="4"/>
+      <c r="K45" s="4"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
+      <c r="P45" s="4"/>
+      <c r="Q45" s="4"/>
+    </row>
+    <row r="46" spans="1:17">
       <c r="A46" s="4"/>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -2263,10 +2175,8 @@
       <c r="O46" s="4"/>
       <c r="P46" s="4"/>
       <c r="Q46" s="4"/>
-      <c r="R46" s="4"/>
-      <c r="S46" s="4"/>
-    </row>
-    <row r="47" spans="1:19">
+    </row>
+    <row r="47" spans="1:17">
       <c r="A47" s="4"/>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
@@ -2284,10 +2194,8 @@
       <c r="O47" s="4"/>
       <c r="P47" s="4"/>
       <c r="Q47" s="4"/>
-      <c r="R47" s="4"/>
-      <c r="S47" s="4"/>
-    </row>
-    <row r="48" spans="1:19">
+    </row>
+    <row r="48" spans="1:17">
       <c r="A48" s="4"/>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -2305,10 +2213,8 @@
       <c r="O48" s="4"/>
       <c r="P48" s="4"/>
       <c r="Q48" s="4"/>
-      <c r="R48" s="4"/>
-      <c r="S48" s="4"/>
-    </row>
-    <row r="49" spans="1:19">
+    </row>
+    <row r="49" spans="1:17">
       <c r="A49" s="4"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
@@ -2326,10 +2232,8 @@
       <c r="O49" s="4"/>
       <c r="P49" s="4"/>
       <c r="Q49" s="4"/>
-      <c r="R49" s="4"/>
-      <c r="S49" s="4"/>
-    </row>
-    <row r="50" spans="1:19">
+    </row>
+    <row r="50" spans="1:17">
       <c r="A50" s="4"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
@@ -2347,10 +2251,8 @@
       <c r="O50" s="4"/>
       <c r="P50" s="4"/>
       <c r="Q50" s="4"/>
-      <c r="R50" s="4"/>
-      <c r="S50" s="4"/>
-    </row>
-    <row r="51" spans="1:19">
+    </row>
+    <row r="51" spans="1:17">
       <c r="A51" s="4"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
@@ -2368,10 +2270,8 @@
       <c r="O51" s="4"/>
       <c r="P51" s="4"/>
       <c r="Q51" s="4"/>
-      <c r="R51" s="4"/>
-      <c r="S51" s="4"/>
-    </row>
-    <row r="52" spans="1:19">
+    </row>
+    <row r="52" spans="1:17">
       <c r="A52" s="4"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -2389,10 +2289,8 @@
       <c r="O52" s="4"/>
       <c r="P52" s="4"/>
       <c r="Q52" s="4"/>
-      <c r="R52" s="4"/>
-      <c r="S52" s="4"/>
-    </row>
-    <row r="53" spans="1:19">
+    </row>
+    <row r="53" spans="1:17">
       <c r="A53" s="4"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -2410,10 +2308,8 @@
       <c r="O53" s="4"/>
       <c r="P53" s="4"/>
       <c r="Q53" s="4"/>
-      <c r="R53" s="4"/>
-      <c r="S53" s="4"/>
-    </row>
-    <row r="54" spans="1:19">
+    </row>
+    <row r="54" spans="1:17">
       <c r="A54" s="4"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -2431,10 +2327,8 @@
       <c r="O54" s="4"/>
       <c r="P54" s="4"/>
       <c r="Q54" s="4"/>
-      <c r="R54" s="4"/>
-      <c r="S54" s="4"/>
-    </row>
-    <row r="55" spans="1:19">
+    </row>
+    <row r="55" spans="1:17">
       <c r="A55" s="4"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -2452,10 +2346,8 @@
       <c r="O55" s="4"/>
       <c r="P55" s="4"/>
       <c r="Q55" s="4"/>
-      <c r="R55" s="4"/>
-      <c r="S55" s="4"/>
-    </row>
-    <row r="56" spans="1:19">
+    </row>
+    <row r="56" spans="1:17">
       <c r="A56" s="4"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -2473,10 +2365,8 @@
       <c r="O56" s="4"/>
       <c r="P56" s="4"/>
       <c r="Q56" s="4"/>
-      <c r="R56" s="4"/>
-      <c r="S56" s="4"/>
-    </row>
-    <row r="57" spans="1:19">
+    </row>
+    <row r="57" spans="1:17">
       <c r="A57" s="4"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
@@ -2494,10 +2384,8 @@
       <c r="O57" s="4"/>
       <c r="P57" s="4"/>
       <c r="Q57" s="4"/>
-      <c r="R57" s="4"/>
-      <c r="S57" s="4"/>
-    </row>
-    <row r="58" spans="1:19">
+    </row>
+    <row r="58" spans="1:17">
       <c r="A58" s="4"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -2515,10 +2403,8 @@
       <c r="O58" s="4"/>
       <c r="P58" s="4"/>
       <c r="Q58" s="4"/>
-      <c r="R58" s="4"/>
-      <c r="S58" s="4"/>
-    </row>
-    <row r="59" spans="1:19">
+    </row>
+    <row r="59" spans="1:17">
       <c r="A59" s="4"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -2536,10 +2422,8 @@
       <c r="O59" s="4"/>
       <c r="P59" s="4"/>
       <c r="Q59" s="4"/>
-      <c r="R59" s="4"/>
-      <c r="S59" s="4"/>
-    </row>
-    <row r="60" spans="1:19">
+    </row>
+    <row r="60" spans="1:17">
       <c r="A60" s="4"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -2557,10 +2441,8 @@
       <c r="O60" s="4"/>
       <c r="P60" s="4"/>
       <c r="Q60" s="4"/>
-      <c r="R60" s="4"/>
-      <c r="S60" s="4"/>
-    </row>
-    <row r="61" spans="1:19">
+    </row>
+    <row r="61" spans="1:17">
       <c r="A61" s="4"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
@@ -2578,10 +2460,8 @@
       <c r="O61" s="4"/>
       <c r="P61" s="4"/>
       <c r="Q61" s="4"/>
-      <c r="R61" s="4"/>
-      <c r="S61" s="4"/>
-    </row>
-    <row r="62" spans="1:19">
+    </row>
+    <row r="62" spans="1:17">
       <c r="A62" s="4"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -2599,10 +2479,8 @@
       <c r="O62" s="4"/>
       <c r="P62" s="4"/>
       <c r="Q62" s="4"/>
-      <c r="R62" s="4"/>
-      <c r="S62" s="4"/>
-    </row>
-    <row r="63" spans="1:19">
+    </row>
+    <row r="63" spans="1:17">
       <c r="A63" s="4"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -2620,10 +2498,8 @@
       <c r="O63" s="4"/>
       <c r="P63" s="4"/>
       <c r="Q63" s="4"/>
-      <c r="R63" s="4"/>
-      <c r="S63" s="4"/>
-    </row>
-    <row r="64" spans="1:19">
+    </row>
+    <row r="64" spans="1:17">
       <c r="A64" s="4"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -2641,10 +2517,8 @@
       <c r="O64" s="4"/>
       <c r="P64" s="4"/>
       <c r="Q64" s="4"/>
-      <c r="R64" s="4"/>
-      <c r="S64" s="4"/>
-    </row>
-    <row r="65" spans="1:19">
+    </row>
+    <row r="65" spans="1:17">
       <c r="A65" s="4"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -2662,10 +2536,8 @@
       <c r="O65" s="4"/>
       <c r="P65" s="4"/>
       <c r="Q65" s="4"/>
-      <c r="R65" s="4"/>
-      <c r="S65" s="4"/>
-    </row>
-    <row r="66" spans="1:19">
+    </row>
+    <row r="66" spans="1:17">
       <c r="A66" s="4"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -2683,10 +2555,8 @@
       <c r="O66" s="4"/>
       <c r="P66" s="4"/>
       <c r="Q66" s="4"/>
-      <c r="R66" s="4"/>
-      <c r="S66" s="4"/>
-    </row>
-    <row r="67" spans="1:19">
+    </row>
+    <row r="67" spans="1:17">
       <c r="A67" s="4"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
@@ -2704,10 +2574,8 @@
       <c r="O67" s="4"/>
       <c r="P67" s="4"/>
       <c r="Q67" s="4"/>
-      <c r="R67" s="4"/>
-      <c r="S67" s="4"/>
-    </row>
-    <row r="68" spans="1:19">
+    </row>
+    <row r="68" spans="1:17">
       <c r="A68" s="4"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
@@ -2725,10 +2593,8 @@
       <c r="O68" s="4"/>
       <c r="P68" s="4"/>
       <c r="Q68" s="4"/>
-      <c r="R68" s="4"/>
-      <c r="S68" s="4"/>
-    </row>
-    <row r="69" spans="1:19">
+    </row>
+    <row r="69" spans="1:17">
       <c r="A69" s="4"/>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
@@ -2746,10 +2612,8 @@
       <c r="O69" s="4"/>
       <c r="P69" s="4"/>
       <c r="Q69" s="4"/>
-      <c r="R69" s="4"/>
-      <c r="S69" s="4"/>
-    </row>
-    <row r="70" spans="1:19">
+    </row>
+    <row r="70" spans="1:17">
       <c r="A70" s="4"/>
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
@@ -2767,10 +2631,8 @@
       <c r="O70" s="4"/>
       <c r="P70" s="4"/>
       <c r="Q70" s="4"/>
-      <c r="R70" s="4"/>
-      <c r="S70" s="4"/>
-    </row>
-    <row r="71" spans="1:19">
+    </row>
+    <row r="71" spans="1:17">
       <c r="A71" s="4"/>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
@@ -2788,10 +2650,8 @@
       <c r="O71" s="4"/>
       <c r="P71" s="4"/>
       <c r="Q71" s="4"/>
-      <c r="R71" s="4"/>
-      <c r="S71" s="4"/>
-    </row>
-    <row r="72" spans="1:19">
+    </row>
+    <row r="72" spans="1:17">
       <c r="A72" s="4"/>
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
@@ -2809,10 +2669,8 @@
       <c r="O72" s="4"/>
       <c r="P72" s="4"/>
       <c r="Q72" s="4"/>
-      <c r="R72" s="4"/>
-      <c r="S72" s="4"/>
-    </row>
-    <row r="73" spans="1:19">
+    </row>
+    <row r="73" spans="1:17">
       <c r="A73" s="4"/>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
@@ -2830,10 +2688,8 @@
       <c r="O73" s="4"/>
       <c r="P73" s="4"/>
       <c r="Q73" s="4"/>
-      <c r="R73" s="4"/>
-      <c r="S73" s="4"/>
-    </row>
-    <row r="74" spans="1:19">
+    </row>
+    <row r="74" spans="1:17">
       <c r="A74" s="4"/>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
@@ -2851,10 +2707,8 @@
       <c r="O74" s="4"/>
       <c r="P74" s="4"/>
       <c r="Q74" s="4"/>
-      <c r="R74" s="4"/>
-      <c r="S74" s="4"/>
-    </row>
-    <row r="75" spans="1:19">
+    </row>
+    <row r="75" spans="1:17">
       <c r="A75" s="4"/>
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
@@ -2872,10 +2726,8 @@
       <c r="O75" s="4"/>
       <c r="P75" s="4"/>
       <c r="Q75" s="4"/>
-      <c r="R75" s="4"/>
-      <c r="S75" s="4"/>
-    </row>
-    <row r="76" spans="1:19">
+    </row>
+    <row r="76" spans="1:17">
       <c r="A76" s="4"/>
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
@@ -2893,10 +2745,8 @@
       <c r="O76" s="4"/>
       <c r="P76" s="4"/>
       <c r="Q76" s="4"/>
-      <c r="R76" s="4"/>
-      <c r="S76" s="4"/>
-    </row>
-    <row r="77" spans="1:19">
+    </row>
+    <row r="77" spans="1:17">
       <c r="A77" s="4"/>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
@@ -2914,10 +2764,8 @@
       <c r="O77" s="4"/>
       <c r="P77" s="4"/>
       <c r="Q77" s="4"/>
-      <c r="R77" s="4"/>
-      <c r="S77" s="4"/>
-    </row>
-    <row r="78" spans="1:19">
+    </row>
+    <row r="78" spans="1:17">
       <c r="A78" s="4"/>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
@@ -2935,10 +2783,8 @@
       <c r="O78" s="4"/>
       <c r="P78" s="4"/>
       <c r="Q78" s="4"/>
-      <c r="R78" s="4"/>
-      <c r="S78" s="4"/>
-    </row>
-    <row r="79" spans="1:19">
+    </row>
+    <row r="79" spans="1:17">
       <c r="A79" s="4"/>
       <c r="B79" s="4"/>
       <c r="C79" s="4"/>
@@ -2956,10 +2802,8 @@
       <c r="O79" s="4"/>
       <c r="P79" s="4"/>
       <c r="Q79" s="4"/>
-      <c r="R79" s="4"/>
-      <c r="S79" s="4"/>
-    </row>
-    <row r="80" spans="1:19">
+    </row>
+    <row r="80" spans="1:17">
       <c r="A80" s="4"/>
       <c r="B80" s="4"/>
       <c r="C80" s="4"/>
@@ -2977,10 +2821,8 @@
       <c r="O80" s="4"/>
       <c r="P80" s="4"/>
       <c r="Q80" s="4"/>
-      <c r="R80" s="4"/>
-      <c r="S80" s="4"/>
-    </row>
-    <row r="81" spans="1:19">
+    </row>
+    <row r="81" spans="1:17">
       <c r="A81" s="4"/>
       <c r="B81" s="4"/>
       <c r="C81" s="4"/>
@@ -2998,10 +2840,8 @@
       <c r="O81" s="4"/>
       <c r="P81" s="4"/>
       <c r="Q81" s="4"/>
-      <c r="R81" s="4"/>
-      <c r="S81" s="4"/>
-    </row>
-    <row r="82" spans="1:19">
+    </row>
+    <row r="82" spans="1:17">
       <c r="A82" s="4"/>
       <c r="B82" s="4"/>
       <c r="C82" s="4"/>
@@ -3019,10 +2859,8 @@
       <c r="O82" s="4"/>
       <c r="P82" s="4"/>
       <c r="Q82" s="4"/>
-      <c r="R82" s="4"/>
-      <c r="S82" s="4"/>
-    </row>
-    <row r="83" spans="1:19">
+    </row>
+    <row r="83" spans="1:17">
       <c r="A83" s="4"/>
       <c r="B83" s="4"/>
       <c r="C83" s="4"/>
@@ -3040,10 +2878,8 @@
       <c r="O83" s="4"/>
       <c r="P83" s="4"/>
       <c r="Q83" s="4"/>
-      <c r="R83" s="4"/>
-      <c r="S83" s="4"/>
-    </row>
-    <row r="84" spans="1:19">
+    </row>
+    <row r="84" spans="1:17">
       <c r="A84" s="4"/>
       <c r="B84" s="4"/>
       <c r="C84" s="4"/>
@@ -3061,10 +2897,8 @@
       <c r="O84" s="4"/>
       <c r="P84" s="4"/>
       <c r="Q84" s="4"/>
-      <c r="R84" s="4"/>
-      <c r="S84" s="4"/>
-    </row>
-    <row r="85" spans="1:19">
+    </row>
+    <row r="85" spans="1:17">
       <c r="A85" s="4"/>
       <c r="B85" s="4"/>
       <c r="C85" s="4"/>
@@ -3082,10 +2916,8 @@
       <c r="O85" s="4"/>
       <c r="P85" s="4"/>
       <c r="Q85" s="4"/>
-      <c r="R85" s="4"/>
-      <c r="S85" s="4"/>
-    </row>
-    <row r="86" spans="1:19">
+    </row>
+    <row r="86" spans="1:17">
       <c r="A86" s="4"/>
       <c r="B86" s="4"/>
       <c r="C86" s="4"/>
@@ -3103,10 +2935,8 @@
       <c r="O86" s="4"/>
       <c r="P86" s="4"/>
       <c r="Q86" s="4"/>
-      <c r="R86" s="4"/>
-      <c r="S86" s="4"/>
-    </row>
-    <row r="87" spans="1:19">
+    </row>
+    <row r="87" spans="1:17">
       <c r="A87" s="4"/>
       <c r="B87" s="4"/>
       <c r="C87" s="4"/>
@@ -3124,10 +2954,8 @@
       <c r="O87" s="4"/>
       <c r="P87" s="4"/>
       <c r="Q87" s="4"/>
-      <c r="R87" s="4"/>
-      <c r="S87" s="4"/>
-    </row>
-    <row r="88" spans="1:19">
+    </row>
+    <row r="88" spans="1:17">
       <c r="A88" s="4"/>
       <c r="B88" s="4"/>
       <c r="C88" s="4"/>
@@ -3145,10 +2973,8 @@
       <c r="O88" s="4"/>
       <c r="P88" s="4"/>
       <c r="Q88" s="4"/>
-      <c r="R88" s="4"/>
-      <c r="S88" s="4"/>
-    </row>
-    <row r="89" spans="1:19">
+    </row>
+    <row r="89" spans="1:17">
       <c r="A89" s="4"/>
       <c r="B89" s="4"/>
       <c r="C89" s="4"/>
@@ -3166,10 +2992,8 @@
       <c r="O89" s="4"/>
       <c r="P89" s="4"/>
       <c r="Q89" s="4"/>
-      <c r="R89" s="4"/>
-      <c r="S89" s="4"/>
-    </row>
-    <row r="90" spans="1:19">
+    </row>
+    <row r="90" spans="1:17">
       <c r="A90" s="4"/>
       <c r="B90" s="4"/>
       <c r="C90" s="4"/>
@@ -3187,10 +3011,8 @@
       <c r="O90" s="4"/>
       <c r="P90" s="4"/>
       <c r="Q90" s="4"/>
-      <c r="R90" s="4"/>
-      <c r="S90" s="4"/>
-    </row>
-    <row r="91" spans="1:19">
+    </row>
+    <row r="91" spans="1:17">
       <c r="A91" s="4"/>
       <c r="B91" s="4"/>
       <c r="C91" s="4"/>
@@ -3208,10 +3030,8 @@
       <c r="O91" s="4"/>
       <c r="P91" s="4"/>
       <c r="Q91" s="4"/>
-      <c r="R91" s="4"/>
-      <c r="S91" s="4"/>
-    </row>
-    <row r="92" spans="1:19">
+    </row>
+    <row r="92" spans="1:17">
       <c r="A92" s="4"/>
       <c r="B92" s="4"/>
       <c r="C92" s="4"/>
@@ -3229,10 +3049,8 @@
       <c r="O92" s="4"/>
       <c r="P92" s="4"/>
       <c r="Q92" s="4"/>
-      <c r="R92" s="4"/>
-      <c r="S92" s="4"/>
-    </row>
-    <row r="93" spans="1:19">
+    </row>
+    <row r="93" spans="1:17">
       <c r="A93" s="4"/>
       <c r="B93" s="4"/>
       <c r="C93" s="4"/>
@@ -3250,10 +3068,8 @@
       <c r="O93" s="4"/>
       <c r="P93" s="4"/>
       <c r="Q93" s="4"/>
-      <c r="R93" s="4"/>
-      <c r="S93" s="4"/>
-    </row>
-    <row r="94" spans="1:19">
+    </row>
+    <row r="94" spans="1:17">
       <c r="A94" s="4"/>
       <c r="B94" s="4"/>
       <c r="C94" s="4"/>
@@ -3271,10 +3087,8 @@
       <c r="O94" s="4"/>
       <c r="P94" s="4"/>
       <c r="Q94" s="4"/>
-      <c r="R94" s="4"/>
-      <c r="S94" s="4"/>
-    </row>
-    <row r="95" spans="1:19">
+    </row>
+    <row r="95" spans="1:17">
       <c r="A95" s="4"/>
       <c r="B95" s="4"/>
       <c r="C95" s="4"/>
@@ -3292,10 +3106,8 @@
       <c r="O95" s="4"/>
       <c r="P95" s="4"/>
       <c r="Q95" s="4"/>
-      <c r="R95" s="4"/>
-      <c r="S95" s="4"/>
-    </row>
-    <row r="96" spans="1:19">
+    </row>
+    <row r="96" spans="1:17">
       <c r="A96" s="4"/>
       <c r="B96" s="4"/>
       <c r="C96" s="4"/>
@@ -3313,10 +3125,8 @@
       <c r="O96" s="4"/>
       <c r="P96" s="4"/>
       <c r="Q96" s="4"/>
-      <c r="R96" s="4"/>
-      <c r="S96" s="4"/>
-    </row>
-    <row r="97" spans="1:19">
+    </row>
+    <row r="97" spans="1:17">
       <c r="A97" s="4"/>
       <c r="B97" s="4"/>
       <c r="C97" s="4"/>
@@ -3334,10 +3144,8 @@
       <c r="O97" s="4"/>
       <c r="P97" s="4"/>
       <c r="Q97" s="4"/>
-      <c r="R97" s="4"/>
-      <c r="S97" s="4"/>
-    </row>
-    <row r="98" spans="1:19">
+    </row>
+    <row r="98" spans="1:17">
       <c r="A98" s="4"/>
       <c r="B98" s="4"/>
       <c r="C98" s="4"/>
@@ -3355,10 +3163,8 @@
       <c r="O98" s="4"/>
       <c r="P98" s="4"/>
       <c r="Q98" s="4"/>
-      <c r="R98" s="4"/>
-      <c r="S98" s="4"/>
-    </row>
-    <row r="99" spans="1:19">
+    </row>
+    <row r="99" spans="1:17">
       <c r="A99" s="4"/>
       <c r="B99" s="4"/>
       <c r="C99" s="4"/>
@@ -3376,10 +3182,8 @@
       <c r="O99" s="4"/>
       <c r="P99" s="4"/>
       <c r="Q99" s="4"/>
-      <c r="R99" s="4"/>
-      <c r="S99" s="4"/>
-    </row>
-    <row r="100" spans="1:19">
+    </row>
+    <row r="100" spans="1:17">
       <c r="A100" s="4"/>
       <c r="B100" s="4"/>
       <c r="C100" s="4"/>
@@ -3397,10 +3201,8 @@
       <c r="O100" s="4"/>
       <c r="P100" s="4"/>
       <c r="Q100" s="4"/>
-      <c r="R100" s="4"/>
-      <c r="S100" s="4"/>
-    </row>
-    <row r="101" spans="1:19">
+    </row>
+    <row r="101" spans="1:17">
       <c r="A101" s="4"/>
       <c r="B101" s="4"/>
       <c r="C101" s="4"/>
@@ -3418,10 +3220,8 @@
       <c r="O101" s="4"/>
       <c r="P101" s="4"/>
       <c r="Q101" s="4"/>
-      <c r="R101" s="4"/>
-      <c r="S101" s="4"/>
-    </row>
-    <row r="102" spans="1:19">
+    </row>
+    <row r="102" spans="1:17">
       <c r="A102" s="4"/>
       <c r="B102" s="4"/>
       <c r="C102" s="4"/>
@@ -3439,10 +3239,8 @@
       <c r="O102" s="4"/>
       <c r="P102" s="4"/>
       <c r="Q102" s="4"/>
-      <c r="R102" s="4"/>
-      <c r="S102" s="4"/>
-    </row>
-    <row r="103" spans="1:19">
+    </row>
+    <row r="103" spans="1:17">
       <c r="A103" s="4"/>
       <c r="B103" s="4"/>
       <c r="C103" s="4"/>
@@ -3460,10 +3258,8 @@
       <c r="O103" s="4"/>
       <c r="P103" s="4"/>
       <c r="Q103" s="4"/>
-      <c r="R103" s="4"/>
-      <c r="S103" s="4"/>
-    </row>
-    <row r="104" spans="1:19">
+    </row>
+    <row r="104" spans="1:17">
       <c r="A104" s="4"/>
       <c r="B104" s="4"/>
       <c r="C104" s="4"/>
@@ -3481,10 +3277,8 @@
       <c r="O104" s="4"/>
       <c r="P104" s="4"/>
       <c r="Q104" s="4"/>
-      <c r="R104" s="4"/>
-      <c r="S104" s="4"/>
-    </row>
-    <row r="105" spans="1:19">
+    </row>
+    <row r="105" spans="1:17">
       <c r="A105" s="4"/>
       <c r="B105" s="4"/>
       <c r="C105" s="4"/>
@@ -3502,10 +3296,8 @@
       <c r="O105" s="4"/>
       <c r="P105" s="4"/>
       <c r="Q105" s="4"/>
-      <c r="R105" s="4"/>
-      <c r="S105" s="4"/>
-    </row>
-    <row r="106" spans="1:19">
+    </row>
+    <row r="106" spans="1:17">
       <c r="A106" s="4"/>
       <c r="B106" s="4"/>
       <c r="C106" s="4"/>
@@ -3523,10 +3315,8 @@
       <c r="O106" s="4"/>
       <c r="P106" s="4"/>
       <c r="Q106" s="4"/>
-      <c r="R106" s="4"/>
-      <c r="S106" s="4"/>
-    </row>
-    <row r="107" spans="1:19">
+    </row>
+    <row r="107" spans="1:17">
       <c r="A107" s="4"/>
       <c r="B107" s="4"/>
       <c r="C107" s="4"/>
@@ -3544,10 +3334,8 @@
       <c r="O107" s="4"/>
       <c r="P107" s="4"/>
       <c r="Q107" s="4"/>
-      <c r="R107" s="4"/>
-      <c r="S107" s="4"/>
-    </row>
-    <row r="108" spans="1:19">
+    </row>
+    <row r="108" spans="1:17">
       <c r="A108" s="4"/>
       <c r="B108" s="4"/>
       <c r="C108" s="4"/>
@@ -3565,10 +3353,8 @@
       <c r="O108" s="4"/>
       <c r="P108" s="4"/>
       <c r="Q108" s="4"/>
-      <c r="R108" s="4"/>
-      <c r="S108" s="4"/>
-    </row>
-    <row r="109" spans="1:19">
+    </row>
+    <row r="109" spans="1:17">
       <c r="A109" s="4"/>
       <c r="B109" s="4"/>
       <c r="C109" s="4"/>
@@ -3586,10 +3372,8 @@
       <c r="O109" s="4"/>
       <c r="P109" s="4"/>
       <c r="Q109" s="4"/>
-      <c r="R109" s="4"/>
-      <c r="S109" s="4"/>
-    </row>
-    <row r="110" spans="1:19">
+    </row>
+    <row r="110" spans="1:17">
       <c r="A110" s="4"/>
       <c r="B110" s="4"/>
       <c r="C110" s="4"/>
@@ -3607,10 +3391,8 @@
       <c r="O110" s="4"/>
       <c r="P110" s="4"/>
       <c r="Q110" s="4"/>
-      <c r="R110" s="4"/>
-      <c r="S110" s="4"/>
-    </row>
-    <row r="111" spans="1:19">
+    </row>
+    <row r="111" spans="1:17">
       <c r="A111" s="4"/>
       <c r="B111" s="4"/>
       <c r="C111" s="4"/>
@@ -3628,10 +3410,8 @@
       <c r="O111" s="4"/>
       <c r="P111" s="4"/>
       <c r="Q111" s="4"/>
-      <c r="R111" s="4"/>
-      <c r="S111" s="4"/>
-    </row>
-    <row r="112" spans="1:19">
+    </row>
+    <row r="112" spans="1:17">
       <c r="A112" s="4"/>
       <c r="B112" s="4"/>
       <c r="C112" s="4"/>
@@ -3649,10 +3429,8 @@
       <c r="O112" s="4"/>
       <c r="P112" s="4"/>
       <c r="Q112" s="4"/>
-      <c r="R112" s="4"/>
-      <c r="S112" s="4"/>
-    </row>
-    <row r="113" spans="1:19">
+    </row>
+    <row r="113" spans="1:17">
       <c r="A113" s="4"/>
       <c r="B113" s="4"/>
       <c r="C113" s="4"/>
@@ -3670,10 +3448,8 @@
       <c r="O113" s="4"/>
       <c r="P113" s="4"/>
       <c r="Q113" s="4"/>
-      <c r="R113" s="4"/>
-      <c r="S113" s="4"/>
-    </row>
-    <row r="114" spans="1:19">
+    </row>
+    <row r="114" spans="1:17">
       <c r="A114" s="4"/>
       <c r="B114" s="4"/>
       <c r="C114" s="4"/>
@@ -3691,10 +3467,8 @@
       <c r="O114" s="4"/>
       <c r="P114" s="4"/>
       <c r="Q114" s="4"/>
-      <c r="R114" s="4"/>
-      <c r="S114" s="4"/>
-    </row>
-    <row r="115" spans="1:19">
+    </row>
+    <row r="115" spans="1:17">
       <c r="A115" s="4"/>
       <c r="B115" s="4"/>
       <c r="C115" s="4"/>
@@ -3712,10 +3486,8 @@
       <c r="O115" s="4"/>
       <c r="P115" s="4"/>
       <c r="Q115" s="4"/>
-      <c r="R115" s="4"/>
-      <c r="S115" s="4"/>
-    </row>
-    <row r="116" spans="1:19">
+    </row>
+    <row r="116" spans="1:17">
       <c r="A116" s="4"/>
       <c r="B116" s="4"/>
       <c r="C116" s="4"/>
@@ -3733,10 +3505,8 @@
       <c r="O116" s="4"/>
       <c r="P116" s="4"/>
       <c r="Q116" s="4"/>
-      <c r="R116" s="4"/>
-      <c r="S116" s="4"/>
-    </row>
-    <row r="117" spans="1:19">
+    </row>
+    <row r="117" spans="1:17">
       <c r="A117" s="4"/>
       <c r="B117" s="4"/>
       <c r="C117" s="4"/>
@@ -3754,10 +3524,8 @@
       <c r="O117" s="4"/>
       <c r="P117" s="4"/>
       <c r="Q117" s="4"/>
-      <c r="R117" s="4"/>
-      <c r="S117" s="4"/>
-    </row>
-    <row r="118" spans="1:19">
+    </row>
+    <row r="118" spans="1:17">
       <c r="A118" s="4"/>
       <c r="B118" s="4"/>
       <c r="C118" s="4"/>
@@ -3775,10 +3543,8 @@
       <c r="O118" s="4"/>
       <c r="P118" s="4"/>
       <c r="Q118" s="4"/>
-      <c r="R118" s="4"/>
-      <c r="S118" s="4"/>
-    </row>
-    <row r="119" spans="1:19">
+    </row>
+    <row r="119" spans="1:17">
       <c r="A119" s="4"/>
       <c r="B119" s="4"/>
       <c r="C119" s="4"/>
@@ -3796,10 +3562,8 @@
       <c r="O119" s="4"/>
       <c r="P119" s="4"/>
       <c r="Q119" s="4"/>
-      <c r="R119" s="4"/>
-      <c r="S119" s="4"/>
-    </row>
-    <row r="120" spans="1:19">
+    </row>
+    <row r="120" spans="1:17">
       <c r="A120" s="4"/>
       <c r="B120" s="4"/>
       <c r="C120" s="4"/>
@@ -3817,10 +3581,8 @@
       <c r="O120" s="4"/>
       <c r="P120" s="4"/>
       <c r="Q120" s="4"/>
-      <c r="R120" s="4"/>
-      <c r="S120" s="4"/>
-    </row>
-    <row r="121" spans="1:19">
+    </row>
+    <row r="121" spans="1:17">
       <c r="A121" s="4"/>
       <c r="B121" s="4"/>
       <c r="C121" s="4"/>
@@ -3838,10 +3600,8 @@
       <c r="O121" s="4"/>
       <c r="P121" s="4"/>
       <c r="Q121" s="4"/>
-      <c r="R121" s="4"/>
-      <c r="S121" s="4"/>
-    </row>
-    <row r="122" spans="1:19">
+    </row>
+    <row r="122" spans="1:17">
       <c r="A122" s="4"/>
       <c r="B122" s="4"/>
       <c r="C122" s="4"/>
@@ -3859,10 +3619,8 @@
       <c r="O122" s="4"/>
       <c r="P122" s="4"/>
       <c r="Q122" s="4"/>
-      <c r="R122" s="4"/>
-      <c r="S122" s="4"/>
-    </row>
-    <row r="123" spans="1:19">
+    </row>
+    <row r="123" spans="1:17">
       <c r="A123" s="4"/>
       <c r="B123" s="4"/>
       <c r="C123" s="4"/>
@@ -3880,10 +3638,8 @@
       <c r="O123" s="4"/>
       <c r="P123" s="4"/>
       <c r="Q123" s="4"/>
-      <c r="R123" s="4"/>
-      <c r="S123" s="4"/>
-    </row>
-    <row r="124" spans="1:19">
+    </row>
+    <row r="124" spans="1:17">
       <c r="A124" s="4"/>
       <c r="B124" s="4"/>
       <c r="C124" s="4"/>
@@ -3901,10 +3657,8 @@
       <c r="O124" s="4"/>
       <c r="P124" s="4"/>
       <c r="Q124" s="4"/>
-      <c r="R124" s="4"/>
-      <c r="S124" s="4"/>
-    </row>
-    <row r="125" spans="1:19">
+    </row>
+    <row r="125" spans="1:17">
       <c r="A125" s="4"/>
       <c r="B125" s="4"/>
       <c r="C125" s="4"/>
@@ -3922,10 +3676,8 @@
       <c r="O125" s="4"/>
       <c r="P125" s="4"/>
       <c r="Q125" s="4"/>
-      <c r="R125" s="4"/>
-      <c r="S125" s="4"/>
-    </row>
-    <row r="126" spans="1:19">
+    </row>
+    <row r="126" spans="1:17">
       <c r="A126" s="4"/>
       <c r="B126" s="4"/>
       <c r="C126" s="4"/>
@@ -3943,10 +3695,8 @@
       <c r="O126" s="4"/>
       <c r="P126" s="4"/>
       <c r="Q126" s="4"/>
-      <c r="R126" s="4"/>
-      <c r="S126" s="4"/>
-    </row>
-    <row r="127" spans="1:19">
+    </row>
+    <row r="127" spans="1:17">
       <c r="A127" s="4"/>
       <c r="B127" s="4"/>
       <c r="C127" s="4"/>
@@ -3964,10 +3714,8 @@
       <c r="O127" s="4"/>
       <c r="P127" s="4"/>
       <c r="Q127" s="4"/>
-      <c r="R127" s="4"/>
-      <c r="S127" s="4"/>
-    </row>
-    <row r="128" spans="1:19">
+    </row>
+    <row r="128" spans="1:17">
       <c r="A128" s="4"/>
       <c r="B128" s="4"/>
       <c r="C128" s="4"/>
@@ -3985,10 +3733,8 @@
       <c r="O128" s="4"/>
       <c r="P128" s="4"/>
       <c r="Q128" s="4"/>
-      <c r="R128" s="4"/>
-      <c r="S128" s="4"/>
-    </row>
-    <row r="129" spans="1:19">
+    </row>
+    <row r="129" spans="1:17">
       <c r="A129" s="4"/>
       <c r="B129" s="4"/>
       <c r="C129" s="4"/>
@@ -4006,10 +3752,8 @@
       <c r="O129" s="4"/>
       <c r="P129" s="4"/>
       <c r="Q129" s="4"/>
-      <c r="R129" s="4"/>
-      <c r="S129" s="4"/>
-    </row>
-    <row r="130" spans="1:19">
+    </row>
+    <row r="130" spans="1:17">
       <c r="A130" s="4"/>
       <c r="B130" s="4"/>
       <c r="C130" s="4"/>
@@ -4027,10 +3771,8 @@
       <c r="O130" s="4"/>
       <c r="P130" s="4"/>
       <c r="Q130" s="4"/>
-      <c r="R130" s="4"/>
-      <c r="S130" s="4"/>
-    </row>
-    <row r="131" spans="1:19">
+    </row>
+    <row r="131" spans="1:17">
       <c r="A131" s="4"/>
       <c r="B131" s="4"/>
       <c r="C131" s="4"/>
@@ -4048,10 +3790,8 @@
       <c r="O131" s="4"/>
       <c r="P131" s="4"/>
       <c r="Q131" s="4"/>
-      <c r="R131" s="4"/>
-      <c r="S131" s="4"/>
-    </row>
-    <row r="132" spans="1:19">
+    </row>
+    <row r="132" spans="1:17">
       <c r="A132" s="4"/>
       <c r="B132" s="4"/>
       <c r="C132" s="4"/>
@@ -4069,10 +3809,8 @@
       <c r="O132" s="4"/>
       <c r="P132" s="4"/>
       <c r="Q132" s="4"/>
-      <c r="R132" s="4"/>
-      <c r="S132" s="4"/>
-    </row>
-    <row r="133" spans="1:19">
+    </row>
+    <row r="133" spans="1:17">
       <c r="A133" s="4"/>
       <c r="B133" s="4"/>
       <c r="C133" s="4"/>
@@ -4090,10 +3828,8 @@
       <c r="O133" s="4"/>
       <c r="P133" s="4"/>
       <c r="Q133" s="4"/>
-      <c r="R133" s="4"/>
-      <c r="S133" s="4"/>
-    </row>
-    <row r="134" spans="1:19">
+    </row>
+    <row r="134" spans="1:17">
       <c r="A134" s="4"/>
       <c r="B134" s="4"/>
       <c r="C134" s="4"/>
@@ -4111,10 +3847,8 @@
       <c r="O134" s="4"/>
       <c r="P134" s="4"/>
       <c r="Q134" s="4"/>
-      <c r="R134" s="4"/>
-      <c r="S134" s="4"/>
-    </row>
-    <row r="135" spans="1:19">
+    </row>
+    <row r="135" spans="1:17">
       <c r="A135" s="4"/>
       <c r="B135" s="4"/>
       <c r="C135" s="4"/>
@@ -4132,10 +3866,8 @@
       <c r="O135" s="4"/>
       <c r="P135" s="4"/>
       <c r="Q135" s="4"/>
-      <c r="R135" s="4"/>
-      <c r="S135" s="4"/>
-    </row>
-    <row r="136" spans="1:19">
+    </row>
+    <row r="136" spans="1:17">
       <c r="A136" s="4"/>
       <c r="B136" s="4"/>
       <c r="C136" s="4"/>
@@ -4153,10 +3885,8 @@
       <c r="O136" s="4"/>
       <c r="P136" s="4"/>
       <c r="Q136" s="4"/>
-      <c r="R136" s="4"/>
-      <c r="S136" s="4"/>
-    </row>
-    <row r="137" spans="1:19">
+    </row>
+    <row r="137" spans="1:17">
       <c r="A137" s="4"/>
       <c r="B137" s="4"/>
       <c r="C137" s="4"/>
@@ -4174,10 +3904,8 @@
       <c r="O137" s="4"/>
       <c r="P137" s="4"/>
       <c r="Q137" s="4"/>
-      <c r="R137" s="4"/>
-      <c r="S137" s="4"/>
-    </row>
-    <row r="138" spans="1:19">
+    </row>
+    <row r="138" spans="1:17">
       <c r="A138" s="4"/>
       <c r="B138" s="4"/>
       <c r="C138" s="4"/>
@@ -4195,10 +3923,8 @@
       <c r="O138" s="4"/>
       <c r="P138" s="4"/>
       <c r="Q138" s="4"/>
-      <c r="R138" s="4"/>
-      <c r="S138" s="4"/>
-    </row>
-    <row r="139" spans="1:19">
+    </row>
+    <row r="139" spans="1:17">
       <c r="A139" s="4"/>
       <c r="B139" s="4"/>
       <c r="C139" s="4"/>
@@ -4216,10 +3942,8 @@
       <c r="O139" s="4"/>
       <c r="P139" s="4"/>
       <c r="Q139" s="4"/>
-      <c r="R139" s="4"/>
-      <c r="S139" s="4"/>
-    </row>
-    <row r="140" spans="1:19">
+    </row>
+    <row r="140" spans="1:17">
       <c r="A140" s="4"/>
       <c r="B140" s="4"/>
       <c r="C140" s="4"/>
@@ -4237,10 +3961,8 @@
       <c r="O140" s="4"/>
       <c r="P140" s="4"/>
       <c r="Q140" s="4"/>
-      <c r="R140" s="4"/>
-      <c r="S140" s="4"/>
-    </row>
-    <row r="141" spans="1:19">
+    </row>
+    <row r="141" spans="1:17">
       <c r="A141" s="4"/>
       <c r="B141" s="4"/>
       <c r="C141" s="4"/>
@@ -4258,10 +3980,8 @@
       <c r="O141" s="4"/>
       <c r="P141" s="4"/>
       <c r="Q141" s="4"/>
-      <c r="R141" s="4"/>
-      <c r="S141" s="4"/>
-    </row>
-    <row r="142" spans="1:19">
+    </row>
+    <row r="142" spans="1:17">
       <c r="A142" s="4"/>
       <c r="B142" s="4"/>
       <c r="C142" s="4"/>
@@ -4279,10 +3999,8 @@
       <c r="O142" s="4"/>
       <c r="P142" s="4"/>
       <c r="Q142" s="4"/>
-      <c r="R142" s="4"/>
-      <c r="S142" s="4"/>
-    </row>
-    <row r="143" spans="1:19">
+    </row>
+    <row r="143" spans="1:17">
       <c r="A143" s="4"/>
       <c r="B143" s="4"/>
       <c r="C143" s="4"/>
@@ -4300,10 +4018,8 @@
       <c r="O143" s="4"/>
       <c r="P143" s="4"/>
       <c r="Q143" s="4"/>
-      <c r="R143" s="4"/>
-      <c r="S143" s="4"/>
-    </row>
-    <row r="144" spans="1:19">
+    </row>
+    <row r="144" spans="1:17">
       <c r="A144" s="4"/>
       <c r="B144" s="4"/>
       <c r="C144" s="4"/>
@@ -4321,10 +4037,8 @@
       <c r="O144" s="4"/>
       <c r="P144" s="4"/>
       <c r="Q144" s="4"/>
-      <c r="R144" s="4"/>
-      <c r="S144" s="4"/>
-    </row>
-    <row r="145" spans="1:19">
+    </row>
+    <row r="145" spans="1:17">
       <c r="A145" s="4"/>
       <c r="B145" s="4"/>
       <c r="C145" s="4"/>
@@ -4342,10 +4056,8 @@
       <c r="O145" s="4"/>
       <c r="P145" s="4"/>
       <c r="Q145" s="4"/>
-      <c r="R145" s="4"/>
-      <c r="S145" s="4"/>
-    </row>
-    <row r="146" spans="1:19">
+    </row>
+    <row r="146" spans="1:17">
       <c r="A146" s="4"/>
       <c r="B146" s="4"/>
       <c r="C146" s="4"/>
@@ -4363,10 +4075,8 @@
       <c r="O146" s="4"/>
       <c r="P146" s="4"/>
       <c r="Q146" s="4"/>
-      <c r="R146" s="4"/>
-      <c r="S146" s="4"/>
-    </row>
-    <row r="147" spans="1:19">
+    </row>
+    <row r="147" spans="1:17">
       <c r="A147" s="4"/>
       <c r="B147" s="4"/>
       <c r="C147" s="4"/>
@@ -4384,10 +4094,8 @@
       <c r="O147" s="4"/>
       <c r="P147" s="4"/>
       <c r="Q147" s="4"/>
-      <c r="R147" s="4"/>
-      <c r="S147" s="4"/>
-    </row>
-    <row r="148" spans="1:19">
+    </row>
+    <row r="148" spans="1:17">
       <c r="A148" s="4"/>
       <c r="B148" s="4"/>
       <c r="C148" s="4"/>
@@ -4405,10 +4113,8 @@
       <c r="O148" s="4"/>
       <c r="P148" s="4"/>
       <c r="Q148" s="4"/>
-      <c r="R148" s="4"/>
-      <c r="S148" s="4"/>
-    </row>
-    <row r="149" spans="1:19">
+    </row>
+    <row r="149" spans="1:17">
       <c r="A149" s="4"/>
       <c r="B149" s="4"/>
       <c r="C149" s="4"/>
@@ -4426,10 +4132,8 @@
       <c r="O149" s="4"/>
       <c r="P149" s="4"/>
       <c r="Q149" s="4"/>
-      <c r="R149" s="4"/>
-      <c r="S149" s="4"/>
-    </row>
-    <row r="150" spans="1:19">
+    </row>
+    <row r="150" spans="1:17">
       <c r="A150" s="4"/>
       <c r="B150" s="4"/>
       <c r="C150" s="4"/>
@@ -4447,10 +4151,8 @@
       <c r="O150" s="4"/>
       <c r="P150" s="4"/>
       <c r="Q150" s="4"/>
-      <c r="R150" s="4"/>
-      <c r="S150" s="4"/>
-    </row>
-    <row r="151" spans="1:19">
+    </row>
+    <row r="151" spans="1:17">
       <c r="A151" s="4"/>
       <c r="B151" s="4"/>
       <c r="C151" s="4"/>
@@ -4468,10 +4170,8 @@
       <c r="O151" s="4"/>
       <c r="P151" s="4"/>
       <c r="Q151" s="4"/>
-      <c r="R151" s="4"/>
-      <c r="S151" s="4"/>
-    </row>
-    <row r="152" spans="1:19">
+    </row>
+    <row r="152" spans="1:17">
       <c r="A152" s="4"/>
       <c r="B152" s="4"/>
       <c r="C152" s="4"/>
@@ -4489,10 +4189,8 @@
       <c r="O152" s="4"/>
       <c r="P152" s="4"/>
       <c r="Q152" s="4"/>
-      <c r="R152" s="4"/>
-      <c r="S152" s="4"/>
-    </row>
-    <row r="153" spans="1:19">
+    </row>
+    <row r="153" spans="1:17">
       <c r="A153" s="4"/>
       <c r="B153" s="4"/>
       <c r="C153" s="4"/>
@@ -4510,10 +4208,8 @@
       <c r="O153" s="4"/>
       <c r="P153" s="4"/>
       <c r="Q153" s="4"/>
-      <c r="R153" s="4"/>
-      <c r="S153" s="4"/>
-    </row>
-    <row r="154" spans="1:19">
+    </row>
+    <row r="154" spans="1:17">
       <c r="A154" s="4"/>
       <c r="B154" s="4"/>
       <c r="C154" s="4"/>
@@ -4531,10 +4227,8 @@
       <c r="O154" s="4"/>
       <c r="P154" s="4"/>
       <c r="Q154" s="4"/>
-      <c r="R154" s="4"/>
-      <c r="S154" s="4"/>
-    </row>
-    <row r="155" spans="1:19">
+    </row>
+    <row r="155" spans="1:17">
       <c r="A155" s="4"/>
       <c r="B155" s="4"/>
       <c r="C155" s="4"/>
@@ -4552,10 +4246,8 @@
       <c r="O155" s="4"/>
       <c r="P155" s="4"/>
       <c r="Q155" s="4"/>
-      <c r="R155" s="4"/>
-      <c r="S155" s="4"/>
-    </row>
-    <row r="156" spans="1:19">
+    </row>
+    <row r="156" spans="1:17">
       <c r="A156" s="4"/>
       <c r="B156" s="4"/>
       <c r="C156" s="4"/>
@@ -4573,10 +4265,8 @@
       <c r="O156" s="4"/>
       <c r="P156" s="4"/>
       <c r="Q156" s="4"/>
-      <c r="R156" s="4"/>
-      <c r="S156" s="4"/>
-    </row>
-    <row r="157" spans="1:19">
+    </row>
+    <row r="157" spans="1:17">
       <c r="A157" s="4"/>
       <c r="B157" s="4"/>
       <c r="C157" s="4"/>
@@ -4594,10 +4284,8 @@
       <c r="O157" s="4"/>
       <c r="P157" s="4"/>
       <c r="Q157" s="4"/>
-      <c r="R157" s="4"/>
-      <c r="S157" s="4"/>
-    </row>
-    <row r="158" spans="1:19">
+    </row>
+    <row r="158" spans="1:17">
       <c r="A158" s="4"/>
       <c r="B158" s="4"/>
       <c r="C158" s="4"/>
@@ -4615,10 +4303,8 @@
       <c r="O158" s="4"/>
       <c r="P158" s="4"/>
       <c r="Q158" s="4"/>
-      <c r="R158" s="4"/>
-      <c r="S158" s="4"/>
-    </row>
-    <row r="159" spans="1:19">
+    </row>
+    <row r="159" spans="1:17">
       <c r="A159" s="4"/>
       <c r="B159" s="4"/>
       <c r="C159" s="4"/>
@@ -4636,10 +4322,8 @@
       <c r="O159" s="4"/>
       <c r="P159" s="4"/>
       <c r="Q159" s="4"/>
-      <c r="R159" s="4"/>
-      <c r="S159" s="4"/>
-    </row>
-    <row r="160" spans="1:19">
+    </row>
+    <row r="160" spans="1:17">
       <c r="A160" s="4"/>
       <c r="B160" s="4"/>
       <c r="C160" s="4"/>
@@ -4657,10 +4341,8 @@
       <c r="O160" s="4"/>
       <c r="P160" s="4"/>
       <c r="Q160" s="4"/>
-      <c r="R160" s="4"/>
-      <c r="S160" s="4"/>
-    </row>
-    <row r="161" spans="1:19">
+    </row>
+    <row r="161" spans="1:17">
       <c r="A161" s="4"/>
       <c r="B161" s="4"/>
       <c r="C161" s="4"/>
@@ -4678,10 +4360,8 @@
       <c r="O161" s="4"/>
       <c r="P161" s="4"/>
       <c r="Q161" s="4"/>
-      <c r="R161" s="4"/>
-      <c r="S161" s="4"/>
-    </row>
-    <row r="162" spans="1:19">
+    </row>
+    <row r="162" spans="1:17">
       <c r="A162" s="4"/>
       <c r="B162" s="4"/>
       <c r="C162" s="4"/>
@@ -4699,10 +4379,8 @@
       <c r="O162" s="4"/>
       <c r="P162" s="4"/>
       <c r="Q162" s="4"/>
-      <c r="R162" s="4"/>
-      <c r="S162" s="4"/>
-    </row>
-    <row r="163" spans="1:19">
+    </row>
+    <row r="163" spans="1:17">
       <c r="A163" s="4"/>
       <c r="B163" s="4"/>
       <c r="C163" s="4"/>
@@ -4720,10 +4398,8 @@
       <c r="O163" s="4"/>
       <c r="P163" s="4"/>
       <c r="Q163" s="4"/>
-      <c r="R163" s="4"/>
-      <c r="S163" s="4"/>
-    </row>
-    <row r="164" spans="1:19">
+    </row>
+    <row r="164" spans="1:17">
       <c r="A164" s="4"/>
       <c r="B164" s="4"/>
       <c r="C164" s="4"/>
@@ -4741,10 +4417,8 @@
       <c r="O164" s="4"/>
       <c r="P164" s="4"/>
       <c r="Q164" s="4"/>
-      <c r="R164" s="4"/>
-      <c r="S164" s="4"/>
-    </row>
-    <row r="165" spans="1:19">
+    </row>
+    <row r="165" spans="1:17">
       <c r="A165" s="4"/>
       <c r="B165" s="4"/>
       <c r="C165" s="4"/>
@@ -4762,10 +4436,8 @@
       <c r="O165" s="4"/>
       <c r="P165" s="4"/>
       <c r="Q165" s="4"/>
-      <c r="R165" s="4"/>
-      <c r="S165" s="4"/>
-    </row>
-    <row r="166" spans="1:19">
+    </row>
+    <row r="166" spans="1:17">
       <c r="A166" s="4"/>
       <c r="B166" s="4"/>
       <c r="C166" s="4"/>
@@ -4783,10 +4455,8 @@
       <c r="O166" s="4"/>
       <c r="P166" s="4"/>
       <c r="Q166" s="4"/>
-      <c r="R166" s="4"/>
-      <c r="S166" s="4"/>
-    </row>
-    <row r="167" spans="1:19">
+    </row>
+    <row r="167" spans="1:17">
       <c r="A167" s="4"/>
       <c r="B167" s="4"/>
       <c r="C167" s="4"/>
@@ -4804,10 +4474,8 @@
       <c r="O167" s="4"/>
       <c r="P167" s="4"/>
       <c r="Q167" s="4"/>
-      <c r="R167" s="4"/>
-      <c r="S167" s="4"/>
-    </row>
-    <row r="168" spans="1:19">
+    </row>
+    <row r="168" spans="1:17">
       <c r="A168" s="4"/>
       <c r="B168" s="4"/>
       <c r="C168" s="4"/>
@@ -4825,10 +4493,8 @@
       <c r="O168" s="4"/>
       <c r="P168" s="4"/>
       <c r="Q168" s="4"/>
-      <c r="R168" s="4"/>
-      <c r="S168" s="4"/>
-    </row>
-    <row r="169" spans="1:19">
+    </row>
+    <row r="169" spans="1:17">
       <c r="A169" s="4"/>
       <c r="B169" s="4"/>
       <c r="C169" s="4"/>
@@ -4846,10 +4512,8 @@
       <c r="O169" s="4"/>
       <c r="P169" s="4"/>
       <c r="Q169" s="4"/>
-      <c r="R169" s="4"/>
-      <c r="S169" s="4"/>
-    </row>
-    <row r="170" spans="1:19">
+    </row>
+    <row r="170" spans="1:17">
       <c r="A170" s="4"/>
       <c r="B170" s="4"/>
       <c r="C170" s="4"/>
@@ -4867,10 +4531,8 @@
       <c r="O170" s="4"/>
       <c r="P170" s="4"/>
       <c r="Q170" s="4"/>
-      <c r="R170" s="4"/>
-      <c r="S170" s="4"/>
-    </row>
-    <row r="171" spans="1:19">
+    </row>
+    <row r="171" spans="1:17">
       <c r="A171" s="4"/>
       <c r="B171" s="4"/>
       <c r="C171" s="4"/>
@@ -4888,10 +4550,8 @@
       <c r="O171" s="4"/>
       <c r="P171" s="4"/>
       <c r="Q171" s="4"/>
-      <c r="R171" s="4"/>
-      <c r="S171" s="4"/>
-    </row>
-    <row r="172" spans="1:19">
+    </row>
+    <row r="172" spans="1:17">
       <c r="A172" s="4"/>
       <c r="B172" s="4"/>
       <c r="C172" s="4"/>
@@ -4909,10 +4569,8 @@
       <c r="O172" s="4"/>
       <c r="P172" s="4"/>
       <c r="Q172" s="4"/>
-      <c r="R172" s="4"/>
-      <c r="S172" s="4"/>
-    </row>
-    <row r="173" spans="1:19">
+    </row>
+    <row r="173" spans="1:17">
       <c r="A173" s="4"/>
       <c r="B173" s="4"/>
       <c r="C173" s="4"/>
@@ -4930,10 +4588,8 @@
       <c r="O173" s="4"/>
       <c r="P173" s="4"/>
       <c r="Q173" s="4"/>
-      <c r="R173" s="4"/>
-      <c r="S173" s="4"/>
-    </row>
-    <row r="174" spans="1:19">
+    </row>
+    <row r="174" spans="1:17">
       <c r="A174" s="4"/>
       <c r="B174" s="4"/>
       <c r="C174" s="4"/>
@@ -4951,10 +4607,8 @@
       <c r="O174" s="4"/>
       <c r="P174" s="4"/>
       <c r="Q174" s="4"/>
-      <c r="R174" s="4"/>
-      <c r="S174" s="4"/>
-    </row>
-    <row r="175" spans="1:19">
+    </row>
+    <row r="175" spans="1:17">
       <c r="A175" s="4"/>
       <c r="B175" s="4"/>
       <c r="C175" s="4"/>
@@ -4972,10 +4626,8 @@
       <c r="O175" s="4"/>
       <c r="P175" s="4"/>
       <c r="Q175" s="4"/>
-      <c r="R175" s="4"/>
-      <c r="S175" s="4"/>
-    </row>
-    <row r="176" spans="1:19">
+    </row>
+    <row r="176" spans="1:17">
       <c r="A176" s="4"/>
       <c r="B176" s="4"/>
       <c r="C176" s="4"/>
@@ -4993,10 +4645,8 @@
       <c r="O176" s="4"/>
       <c r="P176" s="4"/>
       <c r="Q176" s="4"/>
-      <c r="R176" s="4"/>
-      <c r="S176" s="4"/>
-    </row>
-    <row r="177" spans="1:19">
+    </row>
+    <row r="177" spans="1:17">
       <c r="A177" s="4"/>
       <c r="B177" s="4"/>
       <c r="C177" s="4"/>
@@ -5014,10 +4664,8 @@
       <c r="O177" s="4"/>
       <c r="P177" s="4"/>
       <c r="Q177" s="4"/>
-      <c r="R177" s="4"/>
-      <c r="S177" s="4"/>
-    </row>
-    <row r="178" spans="1:19">
+    </row>
+    <row r="178" spans="1:17">
       <c r="A178" s="4"/>
       <c r="B178" s="4"/>
       <c r="C178" s="4"/>
@@ -5035,10 +4683,8 @@
       <c r="O178" s="4"/>
       <c r="P178" s="4"/>
       <c r="Q178" s="4"/>
-      <c r="R178" s="4"/>
-      <c r="S178" s="4"/>
-    </row>
-    <row r="179" spans="1:19">
+    </row>
+    <row r="179" spans="1:17">
       <c r="A179" s="4"/>
       <c r="B179" s="4"/>
       <c r="C179" s="4"/>
@@ -5056,10 +4702,8 @@
       <c r="O179" s="4"/>
       <c r="P179" s="4"/>
       <c r="Q179" s="4"/>
-      <c r="R179" s="4"/>
-      <c r="S179" s="4"/>
-    </row>
-    <row r="180" spans="1:19">
+    </row>
+    <row r="180" spans="1:17">
       <c r="A180" s="4"/>
       <c r="B180" s="4"/>
       <c r="C180" s="4"/>
@@ -5077,10 +4721,8 @@
       <c r="O180" s="4"/>
       <c r="P180" s="4"/>
       <c r="Q180" s="4"/>
-      <c r="R180" s="4"/>
-      <c r="S180" s="4"/>
-    </row>
-    <row r="181" spans="1:19">
+    </row>
+    <row r="181" spans="1:17">
       <c r="A181" s="4"/>
       <c r="B181" s="4"/>
       <c r="C181" s="4"/>
@@ -5098,10 +4740,8 @@
       <c r="O181" s="4"/>
       <c r="P181" s="4"/>
       <c r="Q181" s="4"/>
-      <c r="R181" s="4"/>
-      <c r="S181" s="4"/>
-    </row>
-    <row r="182" spans="1:19">
+    </row>
+    <row r="182" spans="1:17">
       <c r="A182" s="4"/>
       <c r="B182" s="4"/>
       <c r="C182" s="4"/>
@@ -5119,10 +4759,8 @@
       <c r="O182" s="4"/>
       <c r="P182" s="4"/>
       <c r="Q182" s="4"/>
-      <c r="R182" s="4"/>
-      <c r="S182" s="4"/>
-    </row>
-    <row r="183" spans="1:19">
+    </row>
+    <row r="183" spans="1:17">
       <c r="A183" s="4"/>
       <c r="B183" s="4"/>
       <c r="C183" s="4"/>
@@ -5140,10 +4778,8 @@
       <c r="O183" s="4"/>
       <c r="P183" s="4"/>
       <c r="Q183" s="4"/>
-      <c r="R183" s="4"/>
-      <c r="S183" s="4"/>
-    </row>
-    <row r="184" spans="1:19">
+    </row>
+    <row r="184" spans="1:17">
       <c r="A184" s="4"/>
       <c r="B184" s="4"/>
       <c r="C184" s="4"/>
@@ -5161,10 +4797,8 @@
       <c r="O184" s="4"/>
       <c r="P184" s="4"/>
       <c r="Q184" s="4"/>
-      <c r="R184" s="4"/>
-      <c r="S184" s="4"/>
-    </row>
-    <row r="185" spans="1:19">
+    </row>
+    <row r="185" spans="1:17">
       <c r="A185" s="4"/>
       <c r="B185" s="4"/>
       <c r="C185" s="4"/>
@@ -5182,10 +4816,8 @@
       <c r="O185" s="4"/>
       <c r="P185" s="4"/>
       <c r="Q185" s="4"/>
-      <c r="R185" s="4"/>
-      <c r="S185" s="4"/>
-    </row>
-    <row r="186" spans="1:19">
+    </row>
+    <row r="186" spans="1:17">
       <c r="A186" s="4"/>
       <c r="B186" s="4"/>
       <c r="C186" s="4"/>
@@ -5203,10 +4835,8 @@
       <c r="O186" s="4"/>
       <c r="P186" s="4"/>
       <c r="Q186" s="4"/>
-      <c r="R186" s="4"/>
-      <c r="S186" s="4"/>
-    </row>
-    <row r="187" spans="1:19">
+    </row>
+    <row r="187" spans="1:17">
       <c r="A187" s="4"/>
       <c r="B187" s="4"/>
       <c r="C187" s="4"/>
@@ -5224,10 +4854,8 @@
       <c r="O187" s="4"/>
       <c r="P187" s="4"/>
       <c r="Q187" s="4"/>
-      <c r="R187" s="4"/>
-      <c r="S187" s="4"/>
-    </row>
-    <row r="188" spans="1:19">
+    </row>
+    <row r="188" spans="1:17">
       <c r="A188" s="4"/>
       <c r="B188" s="4"/>
       <c r="C188" s="4"/>
@@ -5245,10 +4873,8 @@
       <c r="O188" s="4"/>
       <c r="P188" s="4"/>
       <c r="Q188" s="4"/>
-      <c r="R188" s="4"/>
-      <c r="S188" s="4"/>
-    </row>
-    <row r="189" spans="1:19">
+    </row>
+    <row r="189" spans="1:17">
       <c r="A189" s="4"/>
       <c r="B189" s="4"/>
       <c r="C189" s="4"/>
@@ -5266,10 +4892,8 @@
       <c r="O189" s="4"/>
       <c r="P189" s="4"/>
       <c r="Q189" s="4"/>
-      <c r="R189" s="4"/>
-      <c r="S189" s="4"/>
-    </row>
-    <row r="190" spans="1:19">
+    </row>
+    <row r="190" spans="1:17">
       <c r="A190" s="4"/>
       <c r="B190" s="4"/>
       <c r="C190" s="4"/>
@@ -5287,10 +4911,8 @@
       <c r="O190" s="4"/>
       <c r="P190" s="4"/>
       <c r="Q190" s="4"/>
-      <c r="R190" s="4"/>
-      <c r="S190" s="4"/>
-    </row>
-    <row r="191" spans="1:19">
+    </row>
+    <row r="191" spans="1:17">
       <c r="A191" s="4"/>
       <c r="B191" s="4"/>
       <c r="C191" s="4"/>
@@ -5308,10 +4930,8 @@
       <c r="O191" s="4"/>
       <c r="P191" s="4"/>
       <c r="Q191" s="4"/>
-      <c r="R191" s="4"/>
-      <c r="S191" s="4"/>
-    </row>
-    <row r="192" spans="1:19">
+    </row>
+    <row r="192" spans="1:17">
       <c r="A192" s="4"/>
       <c r="B192" s="4"/>
       <c r="C192" s="4"/>
@@ -5329,10 +4949,8 @@
       <c r="O192" s="4"/>
       <c r="P192" s="4"/>
       <c r="Q192" s="4"/>
-      <c r="R192" s="4"/>
-      <c r="S192" s="4"/>
-    </row>
-    <row r="193" spans="1:19">
+    </row>
+    <row r="193" spans="1:17">
       <c r="A193" s="4"/>
       <c r="B193" s="4"/>
       <c r="C193" s="4"/>
@@ -5350,10 +4968,8 @@
       <c r="O193" s="4"/>
       <c r="P193" s="4"/>
       <c r="Q193" s="4"/>
-      <c r="R193" s="4"/>
-      <c r="S193" s="4"/>
-    </row>
-    <row r="194" spans="1:19">
+    </row>
+    <row r="194" spans="1:17">
       <c r="A194" s="4"/>
       <c r="B194" s="4"/>
       <c r="C194" s="4"/>
@@ -5371,10 +4987,8 @@
       <c r="O194" s="4"/>
       <c r="P194" s="4"/>
       <c r="Q194" s="4"/>
-      <c r="R194" s="4"/>
-      <c r="S194" s="4"/>
-    </row>
-    <row r="195" spans="1:19">
+    </row>
+    <row r="195" spans="1:17">
       <c r="A195" s="4"/>
       <c r="B195" s="4"/>
       <c r="C195" s="4"/>
@@ -5392,10 +5006,8 @@
       <c r="O195" s="4"/>
       <c r="P195" s="4"/>
       <c r="Q195" s="4"/>
-      <c r="R195" s="4"/>
-      <c r="S195" s="4"/>
-    </row>
-    <row r="196" spans="1:19">
+    </row>
+    <row r="196" spans="1:17">
       <c r="A196" s="4"/>
       <c r="B196" s="4"/>
       <c r="C196" s="4"/>
@@ -5413,10 +5025,8 @@
       <c r="O196" s="4"/>
       <c r="P196" s="4"/>
       <c r="Q196" s="4"/>
-      <c r="R196" s="4"/>
-      <c r="S196" s="4"/>
-    </row>
-    <row r="197" spans="1:19">
+    </row>
+    <row r="197" spans="1:17">
       <c r="A197" s="4"/>
       <c r="B197" s="4"/>
       <c r="C197" s="4"/>
@@ -5434,10 +5044,8 @@
       <c r="O197" s="4"/>
       <c r="P197" s="4"/>
       <c r="Q197" s="4"/>
-      <c r="R197" s="4"/>
-      <c r="S197" s="4"/>
-    </row>
-    <row r="198" spans="1:19">
+    </row>
+    <row r="198" spans="1:17">
       <c r="A198" s="4"/>
       <c r="B198" s="4"/>
       <c r="C198" s="4"/>
@@ -5455,10 +5063,8 @@
       <c r="O198" s="4"/>
       <c r="P198" s="4"/>
       <c r="Q198" s="4"/>
-      <c r="R198" s="4"/>
-      <c r="S198" s="4"/>
-    </row>
-    <row r="199" spans="1:19">
+    </row>
+    <row r="199" spans="1:17">
       <c r="A199" s="4"/>
       <c r="B199" s="4"/>
       <c r="C199" s="4"/>
@@ -5476,10 +5082,8 @@
       <c r="O199" s="4"/>
       <c r="P199" s="4"/>
       <c r="Q199" s="4"/>
-      <c r="R199" s="4"/>
-      <c r="S199" s="4"/>
-    </row>
-    <row r="200" spans="1:19">
+    </row>
+    <row r="200" spans="1:17">
       <c r="A200" s="4"/>
       <c r="B200" s="4"/>
       <c r="C200" s="4"/>
@@ -5497,10 +5101,8 @@
       <c r="O200" s="4"/>
       <c r="P200" s="4"/>
       <c r="Q200" s="4"/>
-      <c r="R200" s="4"/>
-      <c r="S200" s="4"/>
-    </row>
-    <row r="201" spans="1:19">
+    </row>
+    <row r="201" spans="1:17">
       <c r="A201" s="4"/>
       <c r="B201" s="4"/>
       <c r="C201" s="4"/>
@@ -5518,10 +5120,8 @@
       <c r="O201" s="4"/>
       <c r="P201" s="4"/>
       <c r="Q201" s="4"/>
-      <c r="R201" s="4"/>
-      <c r="S201" s="4"/>
-    </row>
-    <row r="202" spans="1:19">
+    </row>
+    <row r="202" spans="1:17">
       <c r="A202" s="4"/>
       <c r="B202" s="4"/>
       <c r="C202" s="4"/>
@@ -5539,10 +5139,8 @@
       <c r="O202" s="4"/>
       <c r="P202" s="4"/>
       <c r="Q202" s="4"/>
-      <c r="R202" s="4"/>
-      <c r="S202" s="4"/>
-    </row>
-    <row r="203" spans="1:19">
+    </row>
+    <row r="203" spans="1:17">
       <c r="A203" s="4"/>
       <c r="B203" s="4"/>
       <c r="C203" s="4"/>
@@ -5560,10 +5158,8 @@
       <c r="O203" s="4"/>
       <c r="P203" s="4"/>
       <c r="Q203" s="4"/>
-      <c r="R203" s="4"/>
-      <c r="S203" s="4"/>
-    </row>
-    <row r="204" spans="1:19">
+    </row>
+    <row r="204" spans="1:17">
       <c r="A204" s="4"/>
       <c r="B204" s="4"/>
       <c r="C204" s="4"/>
@@ -5581,10 +5177,8 @@
       <c r="O204" s="4"/>
       <c r="P204" s="4"/>
       <c r="Q204" s="4"/>
-      <c r="R204" s="4"/>
-      <c r="S204" s="4"/>
-    </row>
-    <row r="205" spans="1:19">
+    </row>
+    <row r="205" spans="1:17">
       <c r="A205" s="4"/>
       <c r="B205" s="4"/>
       <c r="C205" s="4"/>
@@ -5602,10 +5196,8 @@
       <c r="O205" s="4"/>
       <c r="P205" s="4"/>
       <c r="Q205" s="4"/>
-      <c r="R205" s="4"/>
-      <c r="S205" s="4"/>
-    </row>
-    <row r="206" spans="1:19">
+    </row>
+    <row r="206" spans="1:17">
       <c r="A206" s="4"/>
       <c r="B206" s="4"/>
       <c r="C206" s="4"/>
@@ -5623,10 +5215,8 @@
       <c r="O206" s="4"/>
       <c r="P206" s="4"/>
       <c r="Q206" s="4"/>
-      <c r="R206" s="4"/>
-      <c r="S206" s="4"/>
-    </row>
-    <row r="207" spans="1:19">
+    </row>
+    <row r="207" spans="1:17">
       <c r="A207" s="4"/>
       <c r="B207" s="4"/>
       <c r="C207" s="4"/>
@@ -5644,10 +5234,8 @@
       <c r="O207" s="4"/>
       <c r="P207" s="4"/>
       <c r="Q207" s="4"/>
-      <c r="R207" s="4"/>
-      <c r="S207" s="4"/>
-    </row>
-    <row r="208" spans="1:19">
+    </row>
+    <row r="208" spans="1:17">
       <c r="A208" s="4"/>
       <c r="B208" s="4"/>
       <c r="C208" s="4"/>
@@ -5665,10 +5253,8 @@
       <c r="O208" s="4"/>
       <c r="P208" s="4"/>
       <c r="Q208" s="4"/>
-      <c r="R208" s="4"/>
-      <c r="S208" s="4"/>
-    </row>
-    <row r="209" spans="1:19">
+    </row>
+    <row r="209" spans="1:17">
       <c r="A209" s="4"/>
       <c r="B209" s="4"/>
       <c r="C209" s="4"/>
@@ -5686,10 +5272,8 @@
       <c r="O209" s="4"/>
       <c r="P209" s="4"/>
       <c r="Q209" s="4"/>
-      <c r="R209" s="4"/>
-      <c r="S209" s="4"/>
-    </row>
-    <row r="210" spans="1:19">
+    </row>
+    <row r="210" spans="1:17">
       <c r="A210" s="4"/>
       <c r="B210" s="4"/>
       <c r="C210" s="4"/>
@@ -5707,10 +5291,8 @@
       <c r="O210" s="4"/>
       <c r="P210" s="4"/>
       <c r="Q210" s="4"/>
-      <c r="R210" s="4"/>
-      <c r="S210" s="4"/>
-    </row>
-    <row r="211" spans="1:19">
+    </row>
+    <row r="211" spans="1:17">
       <c r="A211" s="4"/>
       <c r="B211" s="4"/>
       <c r="C211" s="4"/>
@@ -5728,10 +5310,8 @@
       <c r="O211" s="4"/>
       <c r="P211" s="4"/>
       <c r="Q211" s="4"/>
-      <c r="R211" s="4"/>
-      <c r="S211" s="4"/>
-    </row>
-    <row r="212" spans="1:19">
+    </row>
+    <row r="212" spans="1:17">
       <c r="A212" s="4"/>
       <c r="B212" s="4"/>
       <c r="C212" s="4"/>
@@ -5749,10 +5329,8 @@
       <c r="O212" s="4"/>
       <c r="P212" s="4"/>
       <c r="Q212" s="4"/>
-      <c r="R212" s="4"/>
-      <c r="S212" s="4"/>
-    </row>
-    <row r="213" spans="1:19">
+    </row>
+    <row r="213" spans="1:17">
       <c r="A213" s="4"/>
       <c r="B213" s="4"/>
       <c r="C213" s="4"/>
@@ -5770,10 +5348,8 @@
       <c r="O213" s="4"/>
       <c r="P213" s="4"/>
       <c r="Q213" s="4"/>
-      <c r="R213" s="4"/>
-      <c r="S213" s="4"/>
-    </row>
-    <row r="214" spans="1:19">
+    </row>
+    <row r="214" spans="1:17">
       <c r="A214" s="4"/>
       <c r="B214" s="4"/>
       <c r="C214" s="4"/>
@@ -5791,10 +5367,8 @@
       <c r="O214" s="4"/>
       <c r="P214" s="4"/>
       <c r="Q214" s="4"/>
-      <c r="R214" s="4"/>
-      <c r="S214" s="4"/>
-    </row>
-    <row r="215" spans="1:19">
+    </row>
+    <row r="215" spans="1:17">
       <c r="A215" s="4"/>
       <c r="B215" s="4"/>
       <c r="C215" s="4"/>
@@ -5812,10 +5386,8 @@
       <c r="O215" s="4"/>
       <c r="P215" s="4"/>
       <c r="Q215" s="4"/>
-      <c r="R215" s="4"/>
-      <c r="S215" s="4"/>
-    </row>
-    <row r="216" spans="1:19">
+    </row>
+    <row r="216" spans="1:17">
       <c r="A216" s="4"/>
       <c r="B216" s="4"/>
       <c r="C216" s="4"/>
@@ -5833,10 +5405,8 @@
       <c r="O216" s="4"/>
       <c r="P216" s="4"/>
       <c r="Q216" s="4"/>
-      <c r="R216" s="4"/>
-      <c r="S216" s="4"/>
-    </row>
-    <row r="217" spans="1:19">
+    </row>
+    <row r="217" spans="1:17">
       <c r="A217" s="4"/>
       <c r="B217" s="4"/>
       <c r="C217" s="4"/>
@@ -5854,10 +5424,8 @@
       <c r="O217" s="4"/>
       <c r="P217" s="4"/>
       <c r="Q217" s="4"/>
-      <c r="R217" s="4"/>
-      <c r="S217" s="4"/>
-    </row>
-    <row r="218" spans="1:19">
+    </row>
+    <row r="218" spans="1:17">
       <c r="A218" s="4"/>
       <c r="B218" s="4"/>
       <c r="C218" s="4"/>
@@ -5875,10 +5443,8 @@
       <c r="O218" s="4"/>
       <c r="P218" s="4"/>
       <c r="Q218" s="4"/>
-      <c r="R218" s="4"/>
-      <c r="S218" s="4"/>
-    </row>
-    <row r="219" spans="1:19">
+    </row>
+    <row r="219" spans="1:17">
       <c r="A219" s="4"/>
       <c r="B219" s="4"/>
       <c r="C219" s="4"/>
@@ -5896,10 +5462,8 @@
       <c r="O219" s="4"/>
       <c r="P219" s="4"/>
       <c r="Q219" s="4"/>
-      <c r="R219" s="4"/>
-      <c r="S219" s="4"/>
-    </row>
-    <row r="220" spans="1:19">
+    </row>
+    <row r="220" spans="1:17">
       <c r="A220" s="4"/>
       <c r="B220" s="4"/>
       <c r="C220" s="4"/>
@@ -5917,10 +5481,8 @@
       <c r="O220" s="4"/>
       <c r="P220" s="4"/>
       <c r="Q220" s="4"/>
-      <c r="R220" s="4"/>
-      <c r="S220" s="4"/>
-    </row>
-    <row r="221" spans="1:19">
+    </row>
+    <row r="221" spans="1:17">
       <c r="A221" s="4"/>
       <c r="B221" s="4"/>
       <c r="C221" s="4"/>
@@ -5938,10 +5500,8 @@
       <c r="O221" s="4"/>
       <c r="P221" s="4"/>
       <c r="Q221" s="4"/>
-      <c r="R221" s="4"/>
-      <c r="S221" s="4"/>
-    </row>
-    <row r="222" spans="1:19">
+    </row>
+    <row r="222" spans="1:17">
       <c r="A222" s="4"/>
       <c r="B222" s="4"/>
       <c r="C222" s="4"/>
@@ -5959,10 +5519,8 @@
       <c r="O222" s="4"/>
       <c r="P222" s="4"/>
       <c r="Q222" s="4"/>
-      <c r="R222" s="4"/>
-      <c r="S222" s="4"/>
-    </row>
-    <row r="223" spans="1:19">
+    </row>
+    <row r="223" spans="1:17">
       <c r="A223" s="4"/>
       <c r="B223" s="4"/>
       <c r="C223" s="4"/>
@@ -5980,10 +5538,8 @@
       <c r="O223" s="4"/>
       <c r="P223" s="4"/>
       <c r="Q223" s="4"/>
-      <c r="R223" s="4"/>
-      <c r="S223" s="4"/>
-    </row>
-    <row r="224" spans="1:19">
+    </row>
+    <row r="224" spans="1:17">
       <c r="A224" s="4"/>
       <c r="B224" s="4"/>
       <c r="C224" s="4"/>
@@ -6001,10 +5557,8 @@
       <c r="O224" s="4"/>
       <c r="P224" s="4"/>
       <c r="Q224" s="4"/>
-      <c r="R224" s="4"/>
-      <c r="S224" s="4"/>
-    </row>
-    <row r="225" spans="1:19">
+    </row>
+    <row r="225" spans="1:17">
       <c r="A225" s="4"/>
       <c r="B225" s="4"/>
       <c r="C225" s="4"/>
@@ -6022,10 +5576,8 @@
       <c r="O225" s="4"/>
       <c r="P225" s="4"/>
       <c r="Q225" s="4"/>
-      <c r="R225" s="4"/>
-      <c r="S225" s="4"/>
-    </row>
-    <row r="226" spans="1:19">
+    </row>
+    <row r="226" spans="1:17">
       <c r="A226" s="4"/>
       <c r="B226" s="4"/>
       <c r="C226" s="4"/>
@@ -6043,10 +5595,8 @@
       <c r="O226" s="4"/>
       <c r="P226" s="4"/>
       <c r="Q226" s="4"/>
-      <c r="R226" s="4"/>
-      <c r="S226" s="4"/>
-    </row>
-    <row r="227" spans="1:19">
+    </row>
+    <row r="227" spans="1:17">
       <c r="A227" s="4"/>
       <c r="B227" s="4"/>
       <c r="C227" s="4"/>
@@ -6064,10 +5614,8 @@
       <c r="O227" s="4"/>
       <c r="P227" s="4"/>
       <c r="Q227" s="4"/>
-      <c r="R227" s="4"/>
-      <c r="S227" s="4"/>
-    </row>
-    <row r="228" spans="1:19">
+    </row>
+    <row r="228" spans="1:17">
       <c r="A228" s="4"/>
       <c r="B228" s="4"/>
       <c r="C228" s="4"/>
@@ -6085,10 +5633,8 @@
       <c r="O228" s="4"/>
       <c r="P228" s="4"/>
       <c r="Q228" s="4"/>
-      <c r="R228" s="4"/>
-      <c r="S228" s="4"/>
-    </row>
-    <row r="229" spans="1:19">
+    </row>
+    <row r="229" spans="1:17">
       <c r="A229" s="4"/>
       <c r="B229" s="4"/>
       <c r="C229" s="4"/>
@@ -6106,10 +5652,8 @@
       <c r="O229" s="4"/>
       <c r="P229" s="4"/>
       <c r="Q229" s="4"/>
-      <c r="R229" s="4"/>
-      <c r="S229" s="4"/>
-    </row>
-    <row r="230" spans="1:19">
+    </row>
+    <row r="230" spans="1:17">
       <c r="A230" s="4"/>
       <c r="B230" s="4"/>
       <c r="C230" s="4"/>
@@ -6127,10 +5671,8 @@
       <c r="O230" s="4"/>
       <c r="P230" s="4"/>
       <c r="Q230" s="4"/>
-      <c r="R230" s="4"/>
-      <c r="S230" s="4"/>
-    </row>
-    <row r="231" spans="1:19">
+    </row>
+    <row r="231" spans="1:17">
       <c r="A231" s="4"/>
       <c r="B231" s="4"/>
       <c r="C231" s="4"/>
@@ -6148,10 +5690,8 @@
       <c r="O231" s="4"/>
       <c r="P231" s="4"/>
       <c r="Q231" s="4"/>
-      <c r="R231" s="4"/>
-      <c r="S231" s="4"/>
-    </row>
-    <row r="232" spans="1:19">
+    </row>
+    <row r="232" spans="1:17">
       <c r="A232" s="4"/>
       <c r="B232" s="4"/>
       <c r="C232" s="4"/>
@@ -6169,10 +5709,8 @@
       <c r="O232" s="4"/>
       <c r="P232" s="4"/>
       <c r="Q232" s="4"/>
-      <c r="R232" s="4"/>
-      <c r="S232" s="4"/>
-    </row>
-    <row r="233" spans="1:19">
+    </row>
+    <row r="233" spans="1:17">
       <c r="A233" s="4"/>
       <c r="B233" s="4"/>
       <c r="C233" s="4"/>
@@ -6190,10 +5728,8 @@
       <c r="O233" s="4"/>
       <c r="P233" s="4"/>
       <c r="Q233" s="4"/>
-      <c r="R233" s="4"/>
-      <c r="S233" s="4"/>
-    </row>
-    <row r="234" spans="1:19">
+    </row>
+    <row r="234" spans="1:17">
       <c r="A234" s="4"/>
       <c r="B234" s="4"/>
       <c r="C234" s="4"/>
@@ -6211,10 +5747,8 @@
       <c r="O234" s="4"/>
       <c r="P234" s="4"/>
       <c r="Q234" s="4"/>
-      <c r="R234" s="4"/>
-      <c r="S234" s="4"/>
-    </row>
-    <row r="235" spans="1:19">
+    </row>
+    <row r="235" spans="1:17">
       <c r="A235" s="4"/>
       <c r="B235" s="4"/>
       <c r="C235" s="4"/>
@@ -6232,10 +5766,8 @@
       <c r="O235" s="4"/>
       <c r="P235" s="4"/>
       <c r="Q235" s="4"/>
-      <c r="R235" s="4"/>
-      <c r="S235" s="4"/>
-    </row>
-    <row r="236" spans="1:19">
+    </row>
+    <row r="236" spans="1:17">
       <c r="A236" s="4"/>
       <c r="B236" s="4"/>
       <c r="C236" s="4"/>
@@ -6253,10 +5785,8 @@
       <c r="O236" s="4"/>
       <c r="P236" s="4"/>
       <c r="Q236" s="4"/>
-      <c r="R236" s="4"/>
-      <c r="S236" s="4"/>
-    </row>
-    <row r="237" spans="1:19">
+    </row>
+    <row r="237" spans="1:17">
       <c r="A237" s="4"/>
       <c r="B237" s="4"/>
       <c r="C237" s="4"/>
@@ -6274,10 +5804,8 @@
       <c r="O237" s="4"/>
       <c r="P237" s="4"/>
       <c r="Q237" s="4"/>
-      <c r="R237" s="4"/>
-      <c r="S237" s="4"/>
-    </row>
-    <row r="238" spans="1:19">
+    </row>
+    <row r="238" spans="1:17">
       <c r="A238" s="4"/>
       <c r="B238" s="4"/>
       <c r="C238" s="4"/>
@@ -6295,10 +5823,8 @@
       <c r="O238" s="4"/>
       <c r="P238" s="4"/>
       <c r="Q238" s="4"/>
-      <c r="R238" s="4"/>
-      <c r="S238" s="4"/>
-    </row>
-    <row r="239" spans="1:19">
+    </row>
+    <row r="239" spans="1:17">
       <c r="A239" s="4"/>
       <c r="B239" s="4"/>
       <c r="C239" s="4"/>
@@ -6316,10 +5842,8 @@
       <c r="O239" s="4"/>
       <c r="P239" s="4"/>
       <c r="Q239" s="4"/>
-      <c r="R239" s="4"/>
-      <c r="S239" s="4"/>
-    </row>
-    <row r="240" spans="1:19">
+    </row>
+    <row r="240" spans="1:17">
       <c r="A240" s="4"/>
       <c r="B240" s="4"/>
       <c r="C240" s="4"/>
@@ -6337,10 +5861,8 @@
       <c r="O240" s="4"/>
       <c r="P240" s="4"/>
       <c r="Q240" s="4"/>
-      <c r="R240" s="4"/>
-      <c r="S240" s="4"/>
-    </row>
-    <row r="241" spans="1:19">
+    </row>
+    <row r="241" spans="1:17">
       <c r="A241" s="4"/>
       <c r="B241" s="4"/>
       <c r="C241" s="4"/>
@@ -6358,10 +5880,8 @@
       <c r="O241" s="4"/>
       <c r="P241" s="4"/>
       <c r="Q241" s="4"/>
-      <c r="R241" s="4"/>
-      <c r="S241" s="4"/>
-    </row>
-    <row r="242" spans="1:19">
+    </row>
+    <row r="242" spans="1:17">
       <c r="A242" s="4"/>
       <c r="B242" s="4"/>
       <c r="C242" s="4"/>
@@ -6379,10 +5899,8 @@
       <c r="O242" s="4"/>
       <c r="P242" s="4"/>
       <c r="Q242" s="4"/>
-      <c r="R242" s="4"/>
-      <c r="S242" s="4"/>
-    </row>
-    <row r="243" spans="1:19">
+    </row>
+    <row r="243" spans="1:17">
       <c r="A243" s="4"/>
       <c r="B243" s="4"/>
       <c r="C243" s="4"/>
@@ -6400,10 +5918,8 @@
       <c r="O243" s="4"/>
       <c r="P243" s="4"/>
       <c r="Q243" s="4"/>
-      <c r="R243" s="4"/>
-      <c r="S243" s="4"/>
-    </row>
-    <row r="244" spans="1:19">
+    </row>
+    <row r="244" spans="1:17">
       <c r="A244" s="4"/>
       <c r="B244" s="4"/>
       <c r="C244" s="4"/>
@@ -6421,10 +5937,8 @@
       <c r="O244" s="4"/>
       <c r="P244" s="4"/>
       <c r="Q244" s="4"/>
-      <c r="R244" s="4"/>
-      <c r="S244" s="4"/>
-    </row>
-    <row r="245" spans="1:19">
+    </row>
+    <row r="245" spans="1:17">
       <c r="A245" s="4"/>
       <c r="B245" s="4"/>
       <c r="C245" s="4"/>
@@ -6442,10 +5956,8 @@
       <c r="O245" s="4"/>
       <c r="P245" s="4"/>
       <c r="Q245" s="4"/>
-      <c r="R245" s="4"/>
-      <c r="S245" s="4"/>
-    </row>
-    <row r="246" spans="1:19">
+    </row>
+    <row r="246" spans="1:17">
       <c r="A246" s="4"/>
       <c r="B246" s="4"/>
       <c r="C246" s="4"/>
@@ -6463,10 +5975,8 @@
       <c r="O246" s="4"/>
       <c r="P246" s="4"/>
       <c r="Q246" s="4"/>
-      <c r="R246" s="4"/>
-      <c r="S246" s="4"/>
-    </row>
-    <row r="247" spans="1:19">
+    </row>
+    <row r="247" spans="1:17">
       <c r="A247" s="4"/>
       <c r="B247" s="4"/>
       <c r="C247" s="4"/>
@@ -6484,10 +5994,8 @@
       <c r="O247" s="4"/>
       <c r="P247" s="4"/>
       <c r="Q247" s="4"/>
-      <c r="R247" s="4"/>
-      <c r="S247" s="4"/>
-    </row>
-    <row r="248" spans="1:19">
+    </row>
+    <row r="248" spans="1:17">
       <c r="A248" s="4"/>
       <c r="B248" s="4"/>
       <c r="C248" s="4"/>
@@ -6505,10 +6013,8 @@
       <c r="O248" s="4"/>
       <c r="P248" s="4"/>
       <c r="Q248" s="4"/>
-      <c r="R248" s="4"/>
-      <c r="S248" s="4"/>
-    </row>
-    <row r="249" spans="1:19">
+    </row>
+    <row r="249" spans="1:17">
       <c r="A249" s="4"/>
       <c r="B249" s="4"/>
       <c r="C249" s="4"/>
@@ -6526,10 +6032,8 @@
       <c r="O249" s="4"/>
       <c r="P249" s="4"/>
       <c r="Q249" s="4"/>
-      <c r="R249" s="4"/>
-      <c r="S249" s="4"/>
-    </row>
-    <row r="250" spans="1:19">
+    </row>
+    <row r="250" spans="1:17">
       <c r="A250" s="4"/>
       <c r="B250" s="4"/>
       <c r="C250" s="4"/>
@@ -6547,10 +6051,8 @@
       <c r="O250" s="4"/>
       <c r="P250" s="4"/>
       <c r="Q250" s="4"/>
-      <c r="R250" s="4"/>
-      <c r="S250" s="4"/>
-    </row>
-    <row r="251" spans="1:19">
+    </row>
+    <row r="251" spans="1:17">
       <c r="A251" s="4"/>
       <c r="B251" s="4"/>
       <c r="C251" s="4"/>
@@ -6568,10 +6070,8 @@
       <c r="O251" s="4"/>
       <c r="P251" s="4"/>
       <c r="Q251" s="4"/>
-      <c r="R251" s="4"/>
-      <c r="S251" s="4"/>
-    </row>
-    <row r="252" spans="1:19">
+    </row>
+    <row r="252" spans="1:17">
       <c r="A252" s="4"/>
       <c r="B252" s="4"/>
       <c r="C252" s="4"/>
@@ -6589,10 +6089,8 @@
       <c r="O252" s="4"/>
       <c r="P252" s="4"/>
       <c r="Q252" s="4"/>
-      <c r="R252" s="4"/>
-      <c r="S252" s="4"/>
-    </row>
-    <row r="253" spans="1:19">
+    </row>
+    <row r="253" spans="1:17">
       <c r="A253" s="4"/>
       <c r="B253" s="4"/>
       <c r="C253" s="4"/>
@@ -6610,10 +6108,8 @@
       <c r="O253" s="4"/>
       <c r="P253" s="4"/>
       <c r="Q253" s="4"/>
-      <c r="R253" s="4"/>
-      <c r="S253" s="4"/>
-    </row>
-    <row r="254" spans="1:19">
+    </row>
+    <row r="254" spans="1:17">
       <c r="A254" s="4"/>
       <c r="B254" s="4"/>
       <c r="C254" s="4"/>
@@ -6631,10 +6127,8 @@
       <c r="O254" s="4"/>
       <c r="P254" s="4"/>
       <c r="Q254" s="4"/>
-      <c r="R254" s="4"/>
-      <c r="S254" s="4"/>
-    </row>
-    <row r="255" spans="1:19">
+    </row>
+    <row r="255" spans="1:17">
       <c r="A255" s="4"/>
       <c r="B255" s="4"/>
       <c r="C255" s="4"/>
@@ -6652,10 +6146,8 @@
       <c r="O255" s="4"/>
       <c r="P255" s="4"/>
       <c r="Q255" s="4"/>
-      <c r="R255" s="4"/>
-      <c r="S255" s="4"/>
-    </row>
-    <row r="256" spans="1:19">
+    </row>
+    <row r="256" spans="1:17">
       <c r="A256" s="4"/>
       <c r="B256" s="4"/>
       <c r="C256" s="4"/>
@@ -6673,10 +6165,8 @@
       <c r="O256" s="4"/>
       <c r="P256" s="4"/>
       <c r="Q256" s="4"/>
-      <c r="R256" s="4"/>
-      <c r="S256" s="4"/>
-    </row>
-    <row r="257" spans="1:19">
+    </row>
+    <row r="257" spans="1:17">
       <c r="A257" s="4"/>
       <c r="B257" s="4"/>
       <c r="C257" s="4"/>
@@ -6694,10 +6184,8 @@
       <c r="O257" s="4"/>
       <c r="P257" s="4"/>
       <c r="Q257" s="4"/>
-      <c r="R257" s="4"/>
-      <c r="S257" s="4"/>
-    </row>
-    <row r="258" spans="1:19">
+    </row>
+    <row r="258" spans="1:17">
       <c r="A258" s="4"/>
       <c r="B258" s="4"/>
       <c r="C258" s="4"/>
@@ -6715,10 +6203,8 @@
       <c r="O258" s="4"/>
       <c r="P258" s="4"/>
       <c r="Q258" s="4"/>
-      <c r="R258" s="4"/>
-      <c r="S258" s="4"/>
-    </row>
-    <row r="259" spans="1:19">
+    </row>
+    <row r="259" spans="1:17">
       <c r="A259" s="4"/>
       <c r="B259" s="4"/>
       <c r="C259" s="4"/>
@@ -6736,10 +6222,8 @@
       <c r="O259" s="4"/>
       <c r="P259" s="4"/>
       <c r="Q259" s="4"/>
-      <c r="R259" s="4"/>
-      <c r="S259" s="4"/>
-    </row>
-    <row r="260" spans="1:19">
+    </row>
+    <row r="260" spans="1:17">
       <c r="A260" s="4"/>
       <c r="B260" s="4"/>
       <c r="C260" s="4"/>
@@ -6757,10 +6241,8 @@
       <c r="O260" s="4"/>
       <c r="P260" s="4"/>
       <c r="Q260" s="4"/>
-      <c r="R260" s="4"/>
-      <c r="S260" s="4"/>
-    </row>
-    <row r="261" spans="1:19">
+    </row>
+    <row r="261" spans="1:17">
       <c r="A261" s="4"/>
       <c r="B261" s="4"/>
       <c r="C261" s="4"/>
@@ -6778,10 +6260,8 @@
       <c r="O261" s="4"/>
       <c r="P261" s="4"/>
       <c r="Q261" s="4"/>
-      <c r="R261" s="4"/>
-      <c r="S261" s="4"/>
-    </row>
-    <row r="262" spans="1:19">
+    </row>
+    <row r="262" spans="1:17">
       <c r="A262" s="4"/>
       <c r="B262" s="4"/>
       <c r="C262" s="4"/>
@@ -6799,10 +6279,8 @@
       <c r="O262" s="4"/>
       <c r="P262" s="4"/>
       <c r="Q262" s="4"/>
-      <c r="R262" s="4"/>
-      <c r="S262" s="4"/>
-    </row>
-    <row r="263" spans="1:19">
+    </row>
+    <row r="263" spans="1:17">
       <c r="A263" s="4"/>
       <c r="B263" s="4"/>
       <c r="C263" s="4"/>
@@ -6820,10 +6298,8 @@
       <c r="O263" s="4"/>
       <c r="P263" s="4"/>
       <c r="Q263" s="4"/>
-      <c r="R263" s="4"/>
-      <c r="S263" s="4"/>
-    </row>
-    <row r="264" spans="1:19">
+    </row>
+    <row r="264" spans="1:17">
       <c r="A264" s="4"/>
       <c r="B264" s="4"/>
       <c r="C264" s="4"/>
@@ -6841,10 +6317,8 @@
       <c r="O264" s="4"/>
       <c r="P264" s="4"/>
       <c r="Q264" s="4"/>
-      <c r="R264" s="4"/>
-      <c r="S264" s="4"/>
-    </row>
-    <row r="265" spans="1:19">
+    </row>
+    <row r="265" spans="1:17">
       <c r="A265" s="4"/>
       <c r="B265" s="4"/>
       <c r="C265" s="4"/>
@@ -6862,10 +6336,8 @@
       <c r="O265" s="4"/>
       <c r="P265" s="4"/>
       <c r="Q265" s="4"/>
-      <c r="R265" s="4"/>
-      <c r="S265" s="4"/>
-    </row>
-    <row r="266" spans="1:19">
+    </row>
+    <row r="266" spans="1:17">
       <c r="A266" s="4"/>
       <c r="B266" s="4"/>
       <c r="C266" s="4"/>
@@ -6883,10 +6355,8 @@
       <c r="O266" s="4"/>
       <c r="P266" s="4"/>
       <c r="Q266" s="4"/>
-      <c r="R266" s="4"/>
-      <c r="S266" s="4"/>
-    </row>
-    <row r="267" spans="1:19">
+    </row>
+    <row r="267" spans="1:17">
       <c r="A267" s="4"/>
       <c r="B267" s="4"/>
       <c r="C267" s="4"/>
@@ -6904,10 +6374,8 @@
       <c r="O267" s="4"/>
       <c r="P267" s="4"/>
       <c r="Q267" s="4"/>
-      <c r="R267" s="4"/>
-      <c r="S267" s="4"/>
-    </row>
-    <row r="268" spans="1:19">
+    </row>
+    <row r="268" spans="1:17">
       <c r="A268" s="4"/>
       <c r="B268" s="4"/>
       <c r="C268" s="4"/>
@@ -6925,10 +6393,8 @@
       <c r="O268" s="4"/>
       <c r="P268" s="4"/>
       <c r="Q268" s="4"/>
-      <c r="R268" s="4"/>
-      <c r="S268" s="4"/>
-    </row>
-    <row r="269" spans="1:19">
+    </row>
+    <row r="269" spans="1:17">
       <c r="A269" s="4"/>
       <c r="B269" s="4"/>
       <c r="C269" s="4"/>
@@ -6946,10 +6412,8 @@
       <c r="O269" s="4"/>
       <c r="P269" s="4"/>
       <c r="Q269" s="4"/>
-      <c r="R269" s="4"/>
-      <c r="S269" s="4"/>
-    </row>
-    <row r="270" spans="1:19">
+    </row>
+    <row r="270" spans="1:17">
       <c r="A270" s="4"/>
       <c r="B270" s="4"/>
       <c r="C270" s="4"/>
@@ -6967,10 +6431,8 @@
       <c r="O270" s="4"/>
       <c r="P270" s="4"/>
       <c r="Q270" s="4"/>
-      <c r="R270" s="4"/>
-      <c r="S270" s="4"/>
-    </row>
-    <row r="271" spans="1:19">
+    </row>
+    <row r="271" spans="1:17">
       <c r="A271" s="4"/>
       <c r="B271" s="4"/>
       <c r="C271" s="4"/>
@@ -6988,10 +6450,8 @@
       <c r="O271" s="4"/>
       <c r="P271" s="4"/>
       <c r="Q271" s="4"/>
-      <c r="R271" s="4"/>
-      <c r="S271" s="4"/>
-    </row>
-    <row r="272" spans="1:19">
+    </row>
+    <row r="272" spans="1:17">
       <c r="A272" s="4"/>
       <c r="B272" s="4"/>
       <c r="C272" s="4"/>
@@ -7009,10 +6469,8 @@
       <c r="O272" s="4"/>
       <c r="P272" s="4"/>
       <c r="Q272" s="4"/>
-      <c r="R272" s="4"/>
-      <c r="S272" s="4"/>
-    </row>
-    <row r="273" spans="1:19">
+    </row>
+    <row r="273" spans="1:17">
       <c r="A273" s="4"/>
       <c r="B273" s="4"/>
       <c r="C273" s="4"/>
@@ -7030,10 +6488,8 @@
       <c r="O273" s="4"/>
       <c r="P273" s="4"/>
       <c r="Q273" s="4"/>
-      <c r="R273" s="4"/>
-      <c r="S273" s="4"/>
-    </row>
-    <row r="274" spans="1:19">
+    </row>
+    <row r="274" spans="1:17">
       <c r="A274" s="4"/>
       <c r="B274" s="4"/>
       <c r="C274" s="4"/>
@@ -7051,10 +6507,8 @@
       <c r="O274" s="4"/>
       <c r="P274" s="4"/>
       <c r="Q274" s="4"/>
-      <c r="R274" s="4"/>
-      <c r="S274" s="4"/>
-    </row>
-    <row r="275" spans="1:19">
+    </row>
+    <row r="275" spans="1:17">
       <c r="A275" s="4"/>
       <c r="B275" s="4"/>
       <c r="C275" s="4"/>
@@ -7072,10 +6526,8 @@
       <c r="O275" s="4"/>
       <c r="P275" s="4"/>
       <c r="Q275" s="4"/>
-      <c r="R275" s="4"/>
-      <c r="S275" s="4"/>
-    </row>
-    <row r="276" spans="1:19">
+    </row>
+    <row r="276" spans="1:17">
       <c r="A276" s="4"/>
       <c r="B276" s="4"/>
       <c r="C276" s="4"/>
@@ -7093,10 +6545,8 @@
       <c r="O276" s="4"/>
       <c r="P276" s="4"/>
       <c r="Q276" s="4"/>
-      <c r="R276" s="4"/>
-      <c r="S276" s="4"/>
-    </row>
-    <row r="277" spans="1:19">
+    </row>
+    <row r="277" spans="1:17">
       <c r="A277" s="4"/>
       <c r="B277" s="4"/>
       <c r="C277" s="4"/>
@@ -7114,10 +6564,8 @@
       <c r="O277" s="4"/>
       <c r="P277" s="4"/>
       <c r="Q277" s="4"/>
-      <c r="R277" s="4"/>
-      <c r="S277" s="4"/>
-    </row>
-    <row r="278" spans="1:19">
+    </row>
+    <row r="278" spans="1:17">
       <c r="A278" s="4"/>
       <c r="B278" s="4"/>
       <c r="C278" s="4"/>
@@ -7135,10 +6583,8 @@
       <c r="O278" s="4"/>
       <c r="P278" s="4"/>
       <c r="Q278" s="4"/>
-      <c r="R278" s="4"/>
-      <c r="S278" s="4"/>
-    </row>
-    <row r="279" spans="1:19">
+    </row>
+    <row r="279" spans="1:17">
       <c r="A279" s="4"/>
       <c r="B279" s="4"/>
       <c r="C279" s="4"/>
@@ -7156,10 +6602,8 @@
       <c r="O279" s="4"/>
       <c r="P279" s="4"/>
       <c r="Q279" s="4"/>
-      <c r="R279" s="4"/>
-      <c r="S279" s="4"/>
-    </row>
-    <row r="280" spans="1:19">
+    </row>
+    <row r="280" spans="1:17">
       <c r="A280" s="4"/>
       <c r="B280" s="4"/>
       <c r="C280" s="4"/>
@@ -7177,10 +6621,8 @@
       <c r="O280" s="4"/>
       <c r="P280" s="4"/>
       <c r="Q280" s="4"/>
-      <c r="R280" s="4"/>
-      <c r="S280" s="4"/>
-    </row>
-    <row r="281" spans="1:19">
+    </row>
+    <row r="281" spans="1:17">
       <c r="A281" s="4"/>
       <c r="B281" s="4"/>
       <c r="C281" s="4"/>
@@ -7198,10 +6640,8 @@
       <c r="O281" s="4"/>
       <c r="P281" s="4"/>
       <c r="Q281" s="4"/>
-      <c r="R281" s="4"/>
-      <c r="S281" s="4"/>
-    </row>
-    <row r="282" spans="1:19">
+    </row>
+    <row r="282" spans="1:17">
       <c r="A282" s="4"/>
       <c r="B282" s="4"/>
       <c r="C282" s="4"/>
@@ -7219,10 +6659,8 @@
       <c r="O282" s="4"/>
       <c r="P282" s="4"/>
       <c r="Q282" s="4"/>
-      <c r="R282" s="4"/>
-      <c r="S282" s="4"/>
-    </row>
-    <row r="283" spans="1:19">
+    </row>
+    <row r="283" spans="1:17">
       <c r="A283" s="4"/>
       <c r="B283" s="4"/>
       <c r="C283" s="4"/>
@@ -7240,10 +6678,8 @@
       <c r="O283" s="4"/>
       <c r="P283" s="4"/>
       <c r="Q283" s="4"/>
-      <c r="R283" s="4"/>
-      <c r="S283" s="4"/>
-    </row>
-    <row r="284" spans="1:19">
+    </row>
+    <row r="284" spans="1:17">
       <c r="A284" s="4"/>
       <c r="B284" s="4"/>
       <c r="C284" s="4"/>
@@ -7261,10 +6697,8 @@
       <c r="O284" s="4"/>
       <c r="P284" s="4"/>
       <c r="Q284" s="4"/>
-      <c r="R284" s="4"/>
-      <c r="S284" s="4"/>
-    </row>
-    <row r="285" spans="1:19">
+    </row>
+    <row r="285" spans="1:17">
       <c r="A285" s="4"/>
       <c r="B285" s="4"/>
       <c r="C285" s="4"/>
@@ -7282,10 +6716,8 @@
       <c r="O285" s="4"/>
       <c r="P285" s="4"/>
       <c r="Q285" s="4"/>
-      <c r="R285" s="4"/>
-      <c r="S285" s="4"/>
-    </row>
-    <row r="286" spans="1:19">
+    </row>
+    <row r="286" spans="1:17">
       <c r="A286" s="4"/>
       <c r="B286" s="4"/>
       <c r="C286" s="4"/>
@@ -7303,10 +6735,8 @@
       <c r="O286" s="4"/>
       <c r="P286" s="4"/>
       <c r="Q286" s="4"/>
-      <c r="R286" s="4"/>
-      <c r="S286" s="4"/>
-    </row>
-    <row r="287" spans="1:19">
+    </row>
+    <row r="287" spans="1:17">
       <c r="A287" s="4"/>
       <c r="B287" s="4"/>
       <c r="C287" s="4"/>
@@ -7324,10 +6754,8 @@
       <c r="O287" s="4"/>
       <c r="P287" s="4"/>
       <c r="Q287" s="4"/>
-      <c r="R287" s="4"/>
-      <c r="S287" s="4"/>
-    </row>
-    <row r="288" spans="1:19">
+    </row>
+    <row r="288" spans="1:17">
       <c r="A288" s="4"/>
       <c r="B288" s="4"/>
       <c r="C288" s="4"/>
@@ -7345,10 +6773,8 @@
       <c r="O288" s="4"/>
       <c r="P288" s="4"/>
       <c r="Q288" s="4"/>
-      <c r="R288" s="4"/>
-      <c r="S288" s="4"/>
-    </row>
-    <row r="289" spans="1:19">
+    </row>
+    <row r="289" spans="1:17">
       <c r="A289" s="4"/>
       <c r="B289" s="4"/>
       <c r="C289" s="4"/>
@@ -7366,10 +6792,8 @@
       <c r="O289" s="4"/>
       <c r="P289" s="4"/>
       <c r="Q289" s="4"/>
-      <c r="R289" s="4"/>
-      <c r="S289" s="4"/>
-    </row>
-    <row r="290" spans="1:19">
+    </row>
+    <row r="290" spans="1:17">
       <c r="A290" s="4"/>
       <c r="B290" s="4"/>
       <c r="C290" s="4"/>
@@ -7387,10 +6811,8 @@
       <c r="O290" s="4"/>
       <c r="P290" s="4"/>
       <c r="Q290" s="4"/>
-      <c r="R290" s="4"/>
-      <c r="S290" s="4"/>
-    </row>
-    <row r="291" spans="1:19">
+    </row>
+    <row r="291" spans="1:17">
       <c r="A291" s="4"/>
       <c r="B291" s="4"/>
       <c r="C291" s="4"/>
@@ -7408,10 +6830,8 @@
       <c r="O291" s="4"/>
       <c r="P291" s="4"/>
       <c r="Q291" s="4"/>
-      <c r="R291" s="4"/>
-      <c r="S291" s="4"/>
-    </row>
-    <row r="292" spans="1:19">
+    </row>
+    <row r="292" spans="1:17">
       <c r="A292" s="4"/>
       <c r="B292" s="4"/>
       <c r="C292" s="4"/>
@@ -7429,10 +6849,8 @@
       <c r="O292" s="4"/>
       <c r="P292" s="4"/>
       <c r="Q292" s="4"/>
-      <c r="R292" s="4"/>
-      <c r="S292" s="4"/>
-    </row>
-    <row r="293" spans="1:19">
+    </row>
+    <row r="293" spans="1:17">
       <c r="A293" s="4"/>
       <c r="B293" s="4"/>
       <c r="C293" s="4"/>
@@ -7450,10 +6868,8 @@
       <c r="O293" s="4"/>
       <c r="P293" s="4"/>
       <c r="Q293" s="4"/>
-      <c r="R293" s="4"/>
-      <c r="S293" s="4"/>
-    </row>
-    <row r="294" spans="1:19">
+    </row>
+    <row r="294" spans="1:17">
       <c r="A294" s="4"/>
       <c r="B294" s="4"/>
       <c r="C294" s="4"/>
@@ -7471,10 +6887,8 @@
       <c r="O294" s="4"/>
       <c r="P294" s="4"/>
       <c r="Q294" s="4"/>
-      <c r="R294" s="4"/>
-      <c r="S294" s="4"/>
-    </row>
-    <row r="295" spans="1:19">
+    </row>
+    <row r="295" spans="1:17">
       <c r="A295" s="4"/>
       <c r="B295" s="4"/>
       <c r="C295" s="4"/>
@@ -7492,10 +6906,8 @@
       <c r="O295" s="4"/>
       <c r="P295" s="4"/>
       <c r="Q295" s="4"/>
-      <c r="R295" s="4"/>
-      <c r="S295" s="4"/>
-    </row>
-    <row r="296" spans="1:19">
+    </row>
+    <row r="296" spans="1:17">
       <c r="A296" s="4"/>
       <c r="B296" s="4"/>
       <c r="C296" s="4"/>
@@ -7513,10 +6925,8 @@
       <c r="O296" s="4"/>
       <c r="P296" s="4"/>
       <c r="Q296" s="4"/>
-      <c r="R296" s="4"/>
-      <c r="S296" s="4"/>
-    </row>
-    <row r="297" spans="1:19">
+    </row>
+    <row r="297" spans="1:17">
       <c r="A297" s="4"/>
       <c r="B297" s="4"/>
       <c r="C297" s="4"/>
@@ -7534,10 +6944,8 @@
       <c r="O297" s="4"/>
       <c r="P297" s="4"/>
       <c r="Q297" s="4"/>
-      <c r="R297" s="4"/>
-      <c r="S297" s="4"/>
-    </row>
-    <row r="298" spans="1:19">
+    </row>
+    <row r="298" spans="1:17">
       <c r="A298" s="4"/>
       <c r="B298" s="4"/>
       <c r="C298" s="4"/>
@@ -7555,10 +6963,8 @@
       <c r="O298" s="4"/>
       <c r="P298" s="4"/>
       <c r="Q298" s="4"/>
-      <c r="R298" s="4"/>
-      <c r="S298" s="4"/>
-    </row>
-    <row r="299" spans="1:19">
+    </row>
+    <row r="299" spans="1:17">
       <c r="A299" s="4"/>
       <c r="B299" s="4"/>
       <c r="C299" s="4"/>
@@ -7576,10 +6982,8 @@
       <c r="O299" s="4"/>
       <c r="P299" s="4"/>
       <c r="Q299" s="4"/>
-      <c r="R299" s="4"/>
-      <c r="S299" s="4"/>
-    </row>
-    <row r="300" spans="1:19">
+    </row>
+    <row r="300" spans="1:17">
       <c r="A300" s="4"/>
       <c r="B300" s="4"/>
       <c r="C300" s="4"/>
@@ -7597,10 +7001,8 @@
       <c r="O300" s="4"/>
       <c r="P300" s="4"/>
       <c r="Q300" s="4"/>
-      <c r="R300" s="4"/>
-      <c r="S300" s="4"/>
-    </row>
-    <row r="301" spans="1:19">
+    </row>
+    <row r="301" spans="1:17">
       <c r="A301" s="4"/>
       <c r="B301" s="4"/>
       <c r="C301" s="4"/>
@@ -7618,10 +7020,8 @@
       <c r="O301" s="4"/>
       <c r="P301" s="4"/>
       <c r="Q301" s="4"/>
-      <c r="R301" s="4"/>
-      <c r="S301" s="4"/>
-    </row>
-    <row r="302" spans="1:19">
+    </row>
+    <row r="302" spans="1:17">
       <c r="A302" s="4"/>
       <c r="B302" s="4"/>
       <c r="C302" s="4"/>
@@ -7639,10 +7039,8 @@
       <c r="O302" s="4"/>
       <c r="P302" s="4"/>
       <c r="Q302" s="4"/>
-      <c r="R302" s="4"/>
-      <c r="S302" s="4"/>
-    </row>
-    <row r="303" spans="1:19">
+    </row>
+    <row r="303" spans="1:17">
       <c r="A303" s="4"/>
       <c r="B303" s="4"/>
       <c r="C303" s="4"/>
@@ -7660,10 +7058,8 @@
       <c r="O303" s="4"/>
       <c r="P303" s="4"/>
       <c r="Q303" s="4"/>
-      <c r="R303" s="4"/>
-      <c r="S303" s="4"/>
-    </row>
-    <row r="304" spans="1:19">
+    </row>
+    <row r="304" spans="1:17">
       <c r="A304" s="4"/>
       <c r="B304" s="4"/>
       <c r="C304" s="4"/>
@@ -7681,10 +7077,8 @@
       <c r="O304" s="4"/>
       <c r="P304" s="4"/>
       <c r="Q304" s="4"/>
-      <c r="R304" s="4"/>
-      <c r="S304" s="4"/>
-    </row>
-    <row r="305" spans="1:19">
+    </row>
+    <row r="305" spans="1:17">
       <c r="A305" s="4"/>
       <c r="B305" s="4"/>
       <c r="C305" s="4"/>
@@ -7702,10 +7096,8 @@
       <c r="O305" s="4"/>
       <c r="P305" s="4"/>
       <c r="Q305" s="4"/>
-      <c r="R305" s="4"/>
-      <c r="S305" s="4"/>
-    </row>
-    <row r="306" spans="1:19">
+    </row>
+    <row r="306" spans="1:17">
       <c r="A306" s="4"/>
       <c r="B306" s="4"/>
       <c r="C306" s="4"/>
@@ -7723,10 +7115,8 @@
       <c r="O306" s="4"/>
       <c r="P306" s="4"/>
       <c r="Q306" s="4"/>
-      <c r="R306" s="4"/>
-      <c r="S306" s="4"/>
-    </row>
-    <row r="307" spans="1:19">
+    </row>
+    <row r="307" spans="1:17">
       <c r="A307" s="4"/>
       <c r="B307" s="4"/>
       <c r="C307" s="4"/>
@@ -7744,10 +7134,8 @@
       <c r="O307" s="4"/>
       <c r="P307" s="4"/>
       <c r="Q307" s="4"/>
-      <c r="R307" s="4"/>
-      <c r="S307" s="4"/>
-    </row>
-    <row r="308" spans="1:19">
+    </row>
+    <row r="308" spans="1:17">
       <c r="A308" s="4"/>
       <c r="B308" s="4"/>
       <c r="C308" s="4"/>
@@ -7765,10 +7153,8 @@
       <c r="O308" s="4"/>
       <c r="P308" s="4"/>
       <c r="Q308" s="4"/>
-      <c r="R308" s="4"/>
-      <c r="S308" s="4"/>
-    </row>
-    <row r="309" spans="1:19">
+    </row>
+    <row r="309" spans="1:17">
       <c r="A309" s="4"/>
       <c r="B309" s="4"/>
       <c r="C309" s="4"/>
@@ -7786,10 +7172,8 @@
       <c r="O309" s="4"/>
       <c r="P309" s="4"/>
       <c r="Q309" s="4"/>
-      <c r="R309" s="4"/>
-      <c r="S309" s="4"/>
-    </row>
-    <row r="310" spans="1:19">
+    </row>
+    <row r="310" spans="1:17">
       <c r="A310" s="4"/>
       <c r="B310" s="4"/>
       <c r="C310" s="4"/>
@@ -7807,10 +7191,8 @@
       <c r="O310" s="4"/>
       <c r="P310" s="4"/>
       <c r="Q310" s="4"/>
-      <c r="R310" s="4"/>
-      <c r="S310" s="4"/>
-    </row>
-    <row r="311" spans="1:19">
+    </row>
+    <row r="311" spans="1:17">
       <c r="A311" s="4"/>
       <c r="B311" s="4"/>
       <c r="C311" s="4"/>
@@ -7828,10 +7210,8 @@
       <c r="O311" s="4"/>
       <c r="P311" s="4"/>
       <c r="Q311" s="4"/>
-      <c r="R311" s="4"/>
-      <c r="S311" s="4"/>
-    </row>
-    <row r="312" spans="1:19">
+    </row>
+    <row r="312" spans="1:17">
       <c r="A312" s="4"/>
       <c r="B312" s="4"/>
       <c r="C312" s="4"/>
@@ -7849,10 +7229,8 @@
       <c r="O312" s="4"/>
       <c r="P312" s="4"/>
       <c r="Q312" s="4"/>
-      <c r="R312" s="4"/>
-      <c r="S312" s="4"/>
-    </row>
-    <row r="313" spans="1:19">
+    </row>
+    <row r="313" spans="1:17">
       <c r="A313" s="4"/>
       <c r="B313" s="4"/>
       <c r="C313" s="4"/>
@@ -7870,10 +7248,8 @@
       <c r="O313" s="4"/>
       <c r="P313" s="4"/>
       <c r="Q313" s="4"/>
-      <c r="R313" s="4"/>
-      <c r="S313" s="4"/>
-    </row>
-    <row r="314" spans="1:19">
+    </row>
+    <row r="314" spans="1:17">
       <c r="A314" s="4"/>
       <c r="B314" s="4"/>
       <c r="C314" s="4"/>
@@ -7891,10 +7267,8 @@
       <c r="O314" s="4"/>
       <c r="P314" s="4"/>
       <c r="Q314" s="4"/>
-      <c r="R314" s="4"/>
-      <c r="S314" s="4"/>
-    </row>
-    <row r="315" spans="1:19">
+    </row>
+    <row r="315" spans="1:17">
       <c r="A315" s="4"/>
       <c r="B315" s="4"/>
       <c r="C315" s="4"/>
@@ -7912,10 +7286,8 @@
       <c r="O315" s="4"/>
       <c r="P315" s="4"/>
       <c r="Q315" s="4"/>
-      <c r="R315" s="4"/>
-      <c r="S315" s="4"/>
-    </row>
-    <row r="316" spans="1:19">
+    </row>
+    <row r="316" spans="1:17">
       <c r="A316" s="4"/>
       <c r="B316" s="4"/>
       <c r="C316" s="4"/>
@@ -7933,10 +7305,8 @@
       <c r="O316" s="4"/>
       <c r="P316" s="4"/>
       <c r="Q316" s="4"/>
-      <c r="R316" s="4"/>
-      <c r="S316" s="4"/>
-    </row>
-    <row r="317" spans="1:19">
+    </row>
+    <row r="317" spans="1:17">
       <c r="A317" s="4"/>
       <c r="B317" s="4"/>
       <c r="C317" s="4"/>
@@ -7954,10 +7324,8 @@
       <c r="O317" s="4"/>
       <c r="P317" s="4"/>
       <c r="Q317" s="4"/>
-      <c r="R317" s="4"/>
-      <c r="S317" s="4"/>
-    </row>
-    <row r="318" spans="1:19">
+    </row>
+    <row r="318" spans="1:17">
       <c r="A318" s="4"/>
       <c r="B318" s="4"/>
       <c r="C318" s="4"/>
@@ -7975,10 +7343,8 @@
       <c r="O318" s="4"/>
       <c r="P318" s="4"/>
       <c r="Q318" s="4"/>
-      <c r="R318" s="4"/>
-      <c r="S318" s="4"/>
-    </row>
-    <row r="319" spans="1:19">
+    </row>
+    <row r="319" spans="1:17">
       <c r="A319" s="4"/>
       <c r="B319" s="4"/>
       <c r="C319" s="4"/>
@@ -7996,10 +7362,8 @@
       <c r="O319" s="4"/>
       <c r="P319" s="4"/>
       <c r="Q319" s="4"/>
-      <c r="R319" s="4"/>
-      <c r="S319" s="4"/>
-    </row>
-    <row r="320" spans="1:19">
+    </row>
+    <row r="320" spans="1:17">
       <c r="A320" s="4"/>
       <c r="B320" s="4"/>
       <c r="C320" s="4"/>
@@ -8017,10 +7381,8 @@
       <c r="O320" s="4"/>
       <c r="P320" s="4"/>
       <c r="Q320" s="4"/>
-      <c r="R320" s="4"/>
-      <c r="S320" s="4"/>
-    </row>
-    <row r="321" spans="1:19">
+    </row>
+    <row r="321" spans="1:17">
       <c r="A321" s="4"/>
       <c r="B321" s="4"/>
       <c r="C321" s="4"/>
@@ -8038,10 +7400,8 @@
       <c r="O321" s="4"/>
       <c r="P321" s="4"/>
       <c r="Q321" s="4"/>
-      <c r="R321" s="4"/>
-      <c r="S321" s="4"/>
-    </row>
-    <row r="322" spans="1:19">
+    </row>
+    <row r="322" spans="1:17">
       <c r="A322" s="4"/>
       <c r="B322" s="4"/>
       <c r="C322" s="4"/>
@@ -8059,10 +7419,8 @@
       <c r="O322" s="4"/>
       <c r="P322" s="4"/>
       <c r="Q322" s="4"/>
-      <c r="R322" s="4"/>
-      <c r="S322" s="4"/>
-    </row>
-    <row r="323" spans="1:19">
+    </row>
+    <row r="323" spans="1:17">
       <c r="A323" s="4"/>
       <c r="B323" s="4"/>
       <c r="C323" s="4"/>
@@ -8080,10 +7438,8 @@
       <c r="O323" s="4"/>
       <c r="P323" s="4"/>
       <c r="Q323" s="4"/>
-      <c r="R323" s="4"/>
-      <c r="S323" s="4"/>
-    </row>
-    <row r="324" spans="1:19">
+    </row>
+    <row r="324" spans="1:17">
       <c r="A324" s="4"/>
       <c r="B324" s="4"/>
       <c r="C324" s="4"/>
@@ -8101,128 +7457,12 @@
       <c r="O324" s="4"/>
       <c r="P324" s="4"/>
       <c r="Q324" s="4"/>
-      <c r="R324" s="4"/>
-      <c r="S324" s="4"/>
-    </row>
-    <row r="325" spans="1:19">
-      <c r="A325" s="4"/>
-      <c r="B325" s="4"/>
-      <c r="C325" s="4"/>
-      <c r="D325" s="4"/>
-      <c r="E325" s="4"/>
-      <c r="F325" s="4"/>
-      <c r="G325" s="4"/>
-      <c r="H325" s="4"/>
-      <c r="I325" s="4"/>
-      <c r="J325" s="4"/>
-      <c r="K325" s="4"/>
-      <c r="L325" s="4"/>
-      <c r="M325" s="4"/>
-      <c r="N325" s="4"/>
-      <c r="O325" s="4"/>
-      <c r="P325" s="4"/>
-      <c r="Q325" s="4"/>
-      <c r="R325" s="4"/>
-      <c r="S325" s="4"/>
-    </row>
-    <row r="326" spans="1:19">
-      <c r="A326" s="4"/>
-      <c r="B326" s="4"/>
-      <c r="C326" s="4"/>
-      <c r="D326" s="4"/>
-      <c r="E326" s="4"/>
-      <c r="F326" s="4"/>
-      <c r="G326" s="4"/>
-      <c r="H326" s="4"/>
-      <c r="I326" s="4"/>
-      <c r="J326" s="4"/>
-      <c r="K326" s="4"/>
-      <c r="L326" s="4"/>
-      <c r="M326" s="4"/>
-      <c r="N326" s="4"/>
-      <c r="O326" s="4"/>
-      <c r="P326" s="4"/>
-      <c r="Q326" s="4"/>
-      <c r="R326" s="4"/>
-      <c r="S326" s="4"/>
-    </row>
-    <row r="327" spans="1:19">
-      <c r="A327" s="4"/>
-      <c r="B327" s="4"/>
-      <c r="C327" s="4"/>
-      <c r="D327" s="4"/>
-      <c r="E327" s="4"/>
-      <c r="F327" s="4"/>
-      <c r="G327" s="4"/>
-      <c r="H327" s="4"/>
-      <c r="I327" s="4"/>
-      <c r="J327" s="4"/>
-      <c r="K327" s="4"/>
-      <c r="L327" s="4"/>
-      <c r="M327" s="4"/>
-      <c r="N327" s="4"/>
-      <c r="O327" s="4"/>
-      <c r="P327" s="4"/>
-      <c r="Q327" s="4"/>
-      <c r="R327" s="4"/>
-      <c r="S327" s="4"/>
-    </row>
-    <row r="328" spans="1:19">
-      <c r="A328" s="4"/>
-      <c r="B328" s="4"/>
-      <c r="C328" s="4"/>
-      <c r="D328" s="4"/>
-      <c r="E328" s="4"/>
-      <c r="F328" s="4"/>
-      <c r="G328" s="4"/>
-      <c r="H328" s="4"/>
-      <c r="I328" s="4"/>
-      <c r="J328" s="4"/>
-      <c r="K328" s="4"/>
-      <c r="L328" s="4"/>
-      <c r="M328" s="4"/>
-      <c r="N328" s="4"/>
-      <c r="O328" s="4"/>
-      <c r="P328" s="4"/>
-      <c r="Q328" s="4"/>
-      <c r="R328" s="4"/>
-      <c r="S328" s="4"/>
-    </row>
-    <row r="329" spans="1:19">
-      <c r="A329" s="4"/>
-      <c r="B329" s="4"/>
-      <c r="C329" s="4"/>
-      <c r="D329" s="4"/>
-      <c r="E329" s="4"/>
-      <c r="F329" s="4"/>
-      <c r="G329" s="4"/>
-      <c r="H329" s="4"/>
-      <c r="I329" s="4"/>
-      <c r="J329" s="4"/>
-      <c r="K329" s="4"/>
-      <c r="L329" s="4"/>
-      <c r="M329" s="4"/>
-      <c r="N329" s="4"/>
-      <c r="O329" s="4"/>
-      <c r="P329" s="4"/>
-      <c r="Q329" s="4"/>
-      <c r="R329" s="4"/>
-      <c r="S329" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="L31:M31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="L32:M32"/>
+  <mergeCells count="1">
     <mergeCell ref="H34:I34"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="I31:J31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>